<commit_message>
Add NCDOT AADT growth projections and background volumes section
Workbook: new AADT sheet with Page Road count history (stations
0320000269/0320000260), computed CAGRs, selectable 3.0% growth rate,
2028 Build year projections (12,800 vpd south / 8,200 vpd north of
Airport Road), and a difference-method lower-bound estimate for Airport
Road AADT. Memo: new Background Traffic Volumes section and conclusion
updated to reference background volumes. Build year is 2028 per City of
Durham TIA guidelines (conditions one year after completion; 2027
opening assumed).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017bgXFHUDEAABZN3aMvsVWj
</commit_message>
<xml_diff>
--- a/3905_Page_Rd_Trip_Generation/Trip_Generation_3905_Page_Rd_Durham_NC.xlsx
+++ b/3905_Page_Rd_Trip_Generation/Trip_Generation_3905_Page_Rd_Durham_NC.xlsx
@@ -9,9 +9,11 @@
   </bookViews>
   <sheets>
     <sheet name="TripGen" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Dev" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="AADT" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Dev" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
+    <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Area" vbProcedure="false">AADT!$B$2:$J$28</definedName>
     <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">TripGen!$B$2:$K$24</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
@@ -24,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="78">
   <si>
     <t xml:space="preserve">Trip Generation Table - 12th Edition</t>
   </si>
@@ -104,6 +106,102 @@
     <t xml:space="preserve">Result</t>
   </si>
   <si>
+    <t xml:space="preserve">NCDOT AADT Data &amp; Growth Projections - Page Road (SR 1973)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NCDOT AADT History (vpd)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Location (TMS Station)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2013</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2015</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2017</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2019</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2021</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2023¹</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Page Rd south of Airport Rd (0320000269)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Page Rd north of Airport Rd (0320000260)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Growth Rates &amp; Build Year Projection</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Location</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2023 AADT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAGR '13-'23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAGR '17-'23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Selected Rate²</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Build AADT³</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Build AADT (rounded)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Page Rd south of Airport Rd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Page Rd north of Airport Rd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assumed opening year</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Build (analysis) year</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Per City of Durham TIA Guidelines: analysis examines conditions one year after project completion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Airport Road (SR 1971) AADT Estimate - Difference Method</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Page Rd S of Airport Rd minus N of Airport Rd (2023)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Projected to Build year at selected rate (south leg)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. 2023 values are from the NCDOT AADT traffic segment layer (Route 40001973032 = SR 1973/Page Rd; segments MP 3.334-3.620 [TMS 0320000269, AADT 11,000] and MP 2.728-3.334 [TMS 0320000260, AADT 7,100], source "Maintenance"). Earlier years are from the NCDOT AADT station history (ncdot.maps.arcgis.com), retrieved August 2026.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. Selected growth rate is an engineering input (blue). Computed CAGRs bracket it: south leg 5.1% (2013-2023) / 1.8% (2017-2023); north leg -1.2% (2013-2023) / 0.7% (2017-2023). 3.0%/yr compounded is applied corridor-wide as a conservative planning rate.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. Build AADT = 2023 AADT x (1 + selected rate)^(Build year - 2023). Build year per City of Durham TIA Guidelines (durhamnc.gov, "Guidelines for Traffic Impact Analysis (TIA) Requirement"): the analysis must examine expected traffic conditions one year after the project is scheduled to be complete; with an assumed 2027 opening, Build year = 2028.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4. Difference method: the volume change between the two Page Rd legs equals the net traffic exchanged with Airport Rd at the intersection. It is a LOWER-BOUND estimate of Airport Rd AADT - actual Airport Rd AADT = (11,000 + 7,100) - 2 x (Page Rd through volume), which cannot be isolated from AADT data alone. Verify with the project turning movement count.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Development Summary</t>
   </si>
   <si>
@@ -117,9 +215,6 @@
   </si>
   <si>
     <t xml:space="preserve">3905 Page Rd, Durham, NC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Location</t>
   </si>
   <si>
     <t xml:space="preserve">Page Road (SR 1973) at Airport Road (SR 1971)</t>
@@ -171,15 +266,17 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="6">
+  <numFmts count="8">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0&quot; sf&quot;"/>
     <numFmt numFmtId="166" formatCode="#,##0"/>
     <numFmt numFmtId="167" formatCode="0.00"/>
     <numFmt numFmtId="168" formatCode="0%"/>
     <numFmt numFmtId="169" formatCode="General"/>
+    <numFmt numFmtId="170" formatCode="0.0%"/>
+    <numFmt numFmtId="171" formatCode="0"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -237,6 +334,12 @@
     </font>
     <font>
       <i val="true"/>
+      <sz val="9"/>
+      <name val="Segoe UI"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <sz val="9"/>
       <name val="Segoe UI"/>
       <family val="0"/>
@@ -362,11 +465,15 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="39">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -451,20 +558,68 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="11" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="11" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="11" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="11" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="171" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -662,267 +817,267 @@
   <dimension ref="B1:K29"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2.52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="9.52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="39.79"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="7.79"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="6" style="0" width="7.89"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="2.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="9.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="39.79"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="7.79"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="6" style="1" width="7.89"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="2" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1"/>
-      <c r="J2" s="1"/>
-      <c r="K2" s="1"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
+      <c r="J2" s="2"/>
+      <c r="K2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="4" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="F4" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="G4" s="4"/>
-      <c r="H4" s="4"/>
-      <c r="I4" s="5" t="s">
+      <c r="G4" s="5"/>
+      <c r="H4" s="5"/>
+      <c r="I4" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="J4" s="5"/>
-      <c r="K4" s="5"/>
+      <c r="J4" s="6"/>
+      <c r="K4" s="6"/>
     </row>
     <row r="5" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B5" s="2"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="6" t="s">
+      <c r="B5" s="3"/>
+      <c r="C5" s="4"/>
+      <c r="D5" s="4"/>
+      <c r="E5" s="4"/>
+      <c r="F5" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="G5" s="6" t="s">
+      <c r="G5" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="H5" s="6" t="s">
+      <c r="H5" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="I5" s="6" t="s">
+      <c r="I5" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="J5" s="6" t="s">
+      <c r="J5" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="K5" s="7" t="s">
+      <c r="K5" s="8" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B6" s="8" t="s">
+      <c r="B6" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="8"/>
-      <c r="D6" s="8"/>
-      <c r="E6" s="8"/>
-      <c r="F6" s="8"/>
-      <c r="G6" s="8"/>
-      <c r="H6" s="8"/>
-      <c r="I6" s="8"/>
-      <c r="J6" s="8"/>
-      <c r="K6" s="8"/>
+      <c r="C6" s="9"/>
+      <c r="D6" s="9"/>
+      <c r="E6" s="9"/>
+      <c r="F6" s="9"/>
+      <c r="G6" s="9"/>
+      <c r="H6" s="9"/>
+      <c r="I6" s="9"/>
+      <c r="J6" s="9"/>
+      <c r="K6" s="9"/>
     </row>
     <row r="7" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B7" s="9" t="n">
+      <c r="B7" s="10" t="n">
         <v>110</v>
       </c>
-      <c r="C7" s="10" t="s">
+      <c r="C7" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="D7" s="11" t="n">
+      <c r="D7" s="12" t="n">
         <v>150000</v>
       </c>
-      <c r="E7" s="12" t="n">
+      <c r="E7" s="13" t="n">
         <f aca="false">IF(D7&gt;0,ROUND($D$16*(D7/1000),0),0)</f>
         <v>540</v>
       </c>
-      <c r="F7" s="12" t="n">
+      <c r="F7" s="13" t="n">
         <f aca="false">IF(D7&gt;0,ROUND($E$17*H7,0),0)</f>
         <v>62</v>
       </c>
-      <c r="G7" s="12" t="n">
+      <c r="G7" s="13" t="n">
         <f aca="false">H7-F7</f>
         <v>10</v>
       </c>
-      <c r="H7" s="12" t="n">
+      <c r="H7" s="13" t="n">
         <f aca="false">IF(D7&gt;0,ROUND($D$17*(D7/1000),0),0)</f>
         <v>72</v>
       </c>
-      <c r="I7" s="12" t="n">
+      <c r="I7" s="13" t="n">
         <f aca="false">IF(D7&gt;0,ROUND($E$18*K7,0),0)</f>
         <v>18</v>
       </c>
-      <c r="J7" s="12" t="n">
+      <c r="J7" s="13" t="n">
         <f aca="false">K7-I7</f>
         <v>56</v>
       </c>
-      <c r="K7" s="13" t="n">
+      <c r="K7" s="14" t="n">
         <f aca="false">IF(D7&gt;0,ROUND($D$18*(D7/1000),0),0)</f>
         <v>74</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="9" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B9" s="14" t="s">
+      <c r="B9" s="15" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B10" s="14" t="s">
+      <c r="B10" s="15" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B11" s="14" t="s">
+      <c r="B11" s="15" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="13" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="14" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B14" s="15" t="s">
+      <c r="B14" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C14" s="15"/>
-      <c r="D14" s="15"/>
-      <c r="E14" s="15"/>
-      <c r="F14" s="15"/>
+      <c r="C14" s="16"/>
+      <c r="D14" s="16"/>
+      <c r="E14" s="16"/>
+      <c r="F14" s="16"/>
     </row>
     <row r="15" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B15" s="16" t="s">
+      <c r="B15" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="C15" s="16"/>
-      <c r="D15" s="16" t="s">
+      <c r="C15" s="17"/>
+      <c r="D15" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="E15" s="16" t="s">
+      <c r="E15" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="F15" s="16" t="s">
+      <c r="F15" s="17" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B16" s="17" t="s">
+      <c r="B16" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="C16" s="17"/>
-      <c r="D16" s="18" t="n">
+      <c r="C16" s="18"/>
+      <c r="D16" s="19" t="n">
         <v>3.6</v>
       </c>
-      <c r="E16" s="19" t="n">
+      <c r="E16" s="20" t="n">
         <v>0.5</v>
       </c>
-      <c r="F16" s="19" t="n">
+      <c r="F16" s="20" t="n">
         <v>0.5</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B17" s="17" t="s">
+      <c r="B17" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="C17" s="17"/>
-      <c r="D17" s="18" t="n">
+      <c r="C17" s="18"/>
+      <c r="D17" s="19" t="n">
         <v>0.48</v>
       </c>
-      <c r="E17" s="19" t="n">
+      <c r="E17" s="20" t="n">
         <v>0.86</v>
       </c>
-      <c r="F17" s="19" t="n">
+      <c r="F17" s="20" t="n">
         <v>0.14</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B18" s="17" t="s">
+      <c r="B18" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="C18" s="17"/>
-      <c r="D18" s="18" t="n">
+      <c r="C18" s="18"/>
+      <c r="D18" s="19" t="n">
         <v>0.49</v>
       </c>
-      <c r="E18" s="19" t="n">
+      <c r="E18" s="20" t="n">
         <v>0.24</v>
       </c>
-      <c r="F18" s="19" t="n">
+      <c r="F18" s="20" t="n">
         <v>0.76</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B19" s="20" t="s">
+      <c r="B19" s="21" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="21" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B21" s="15" t="s">
+      <c r="B21" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="C21" s="15"/>
-      <c r="D21" s="15"/>
-      <c r="E21" s="15"/>
-      <c r="F21" s="15"/>
+      <c r="C21" s="16"/>
+      <c r="D21" s="16"/>
+      <c r="E21" s="16"/>
+      <c r="F21" s="16"/>
     </row>
     <row r="22" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B22" s="17" t="s">
+      <c r="B22" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="C22" s="17"/>
-      <c r="D22" s="21" t="n">
+      <c r="C22" s="18"/>
+      <c r="D22" s="22" t="n">
         <v>150</v>
       </c>
-      <c r="E22" s="22"/>
-      <c r="F22" s="22"/>
+      <c r="E22" s="23"/>
+      <c r="F22" s="23"/>
     </row>
     <row r="23" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B23" s="17" t="s">
+      <c r="B23" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="C23" s="17"/>
-      <c r="D23" s="23" t="n">
+      <c r="C23" s="18"/>
+      <c r="D23" s="24" t="n">
         <f aca="false">MAX(H7,K7)</f>
         <v>74</v>
       </c>
-      <c r="E23" s="22"/>
-      <c r="F23" s="22"/>
+      <c r="E23" s="23"/>
+      <c r="F23" s="23"/>
     </row>
     <row r="24" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B24" s="17" t="s">
+      <c r="B24" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="C24" s="17"/>
-      <c r="D24" s="16" t="str">
+      <c r="C24" s="18"/>
+      <c r="D24" s="17" t="str">
         <f aca="false">IF(AND(H7&lt;D22,K7&lt;D22),"TIA Not Required","TIA Required")</f>
         <v>TIA Not Required</v>
       </c>
-      <c r="E24" s="16"/>
-      <c r="F24" s="16"/>
+      <c r="E24" s="17"/>
+      <c r="F24" s="17"/>
     </row>
     <row r="25" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="26" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -963,98 +1118,420 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="true"/>
+  </sheetPr>
+  <dimension ref="B2:J28"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="3" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="0" width="13"/>
+  </cols>
+  <sheetData>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B2" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="25"/>
+      <c r="G2" s="25"/>
+      <c r="H2" s="25"/>
+      <c r="I2" s="25"/>
+      <c r="J2" s="25"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B4" s="26" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B5" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" s="17" t="s">
+        <v>29</v>
+      </c>
+      <c r="D5" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="E5" s="17" t="s">
+        <v>31</v>
+      </c>
+      <c r="F5" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="G5" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="H5" s="17" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B6" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="C6" s="27" t="n">
+        <v>6700</v>
+      </c>
+      <c r="D6" s="27" t="n">
+        <v>7700</v>
+      </c>
+      <c r="E6" s="27" t="n">
+        <v>9900</v>
+      </c>
+      <c r="F6" s="24" t="s">
+        <v>36</v>
+      </c>
+      <c r="G6" s="27" t="n">
+        <v>10000</v>
+      </c>
+      <c r="H6" s="27" t="n">
+        <v>11000</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B7" s="18" t="s">
+        <v>37</v>
+      </c>
+      <c r="C7" s="27" t="n">
+        <v>8000</v>
+      </c>
+      <c r="D7" s="27" t="n">
+        <v>5500</v>
+      </c>
+      <c r="E7" s="27" t="n">
+        <v>6800</v>
+      </c>
+      <c r="F7" s="27" t="n">
+        <v>8200</v>
+      </c>
+      <c r="G7" s="27" t="n">
+        <v>6600</v>
+      </c>
+      <c r="H7" s="27" t="n">
+        <v>7100</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B10" s="26" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B11" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="C11" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="D11" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="E11" s="17" t="s">
+        <v>42</v>
+      </c>
+      <c r="F11" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="G11" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="H11" s="17" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B12" s="18" t="s">
+        <v>46</v>
+      </c>
+      <c r="C12" s="28" t="n">
+        <f aca="false">H6</f>
+        <v>11000</v>
+      </c>
+      <c r="D12" s="29" t="n">
+        <f aca="false">(H6/C6)^(1/10)-1</f>
+        <v>0.050828367580992</v>
+      </c>
+      <c r="E12" s="29" t="n">
+        <f aca="false">(H6/E6)^(1/6)-1</f>
+        <v>0.0177151706893666</v>
+      </c>
+      <c r="F12" s="30" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="G12" s="28" t="n">
+        <f aca="false">C12*(1+F12)^($D$16-2023)</f>
+        <v>12752.0148173</v>
+      </c>
+      <c r="H12" s="28" t="n">
+        <f aca="false">ROUND(G12,-2)</f>
+        <v>12800</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B13" s="18" t="s">
+        <v>47</v>
+      </c>
+      <c r="C13" s="28" t="n">
+        <f aca="false">H7</f>
+        <v>7100</v>
+      </c>
+      <c r="D13" s="29" t="n">
+        <f aca="false">(H7/C7)^(1/10)-1</f>
+        <v>-0.0118637399993557</v>
+      </c>
+      <c r="E13" s="29" t="n">
+        <f aca="false">(H7/E7)^(1/6)-1</f>
+        <v>0.0072213107942356</v>
+      </c>
+      <c r="F13" s="30" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="G13" s="28" t="n">
+        <f aca="false">C13*(1+F13)^($D$16-2023)</f>
+        <v>8230.84592753</v>
+      </c>
+      <c r="H13" s="28" t="n">
+        <f aca="false">ROUND(G13,-2)</f>
+        <v>8200</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B15" s="18" t="s">
+        <v>48</v>
+      </c>
+      <c r="C15" s="31"/>
+      <c r="D15" s="32" t="n">
+        <v>2027</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B16" s="18" t="s">
+        <v>49</v>
+      </c>
+      <c r="C16" s="31"/>
+      <c r="D16" s="33" t="n">
+        <f aca="false">D15+1</f>
+        <v>2028</v>
+      </c>
+      <c r="E16" s="34" t="s">
+        <v>50</v>
+      </c>
+      <c r="F16" s="34"/>
+      <c r="G16" s="34"/>
+      <c r="H16" s="34"/>
+      <c r="I16" s="34"/>
+      <c r="J16" s="34"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B19" s="26" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B20" s="18" t="s">
+        <v>52</v>
+      </c>
+      <c r="C20" s="31"/>
+      <c r="D20" s="35" t="n">
+        <f aca="false">C12-C13</f>
+        <v>3900</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B21" s="18" t="s">
+        <v>53</v>
+      </c>
+      <c r="C21" s="31"/>
+      <c r="D21" s="36" t="n">
+        <f aca="false">ROUND(D20*(1+F12)^($D$16-2023),-2)</f>
+        <v>4500</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B24" s="37" t="s">
+        <v>12</v>
+      </c>
+      <c r="C24" s="37"/>
+      <c r="D24" s="37"/>
+      <c r="E24" s="37"/>
+      <c r="F24" s="37"/>
+      <c r="G24" s="37"/>
+      <c r="H24" s="37"/>
+      <c r="I24" s="37"/>
+      <c r="J24" s="37"/>
+    </row>
+    <row r="25" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B25" s="37" t="s">
+        <v>54</v>
+      </c>
+      <c r="C25" s="37"/>
+      <c r="D25" s="37"/>
+      <c r="E25" s="37"/>
+      <c r="F25" s="37"/>
+      <c r="G25" s="37"/>
+      <c r="H25" s="37"/>
+      <c r="I25" s="37"/>
+      <c r="J25" s="37"/>
+    </row>
+    <row r="26" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B26" s="37" t="s">
+        <v>55</v>
+      </c>
+      <c r="C26" s="37"/>
+      <c r="D26" s="37"/>
+      <c r="E26" s="37"/>
+      <c r="F26" s="37"/>
+      <c r="G26" s="37"/>
+      <c r="H26" s="37"/>
+      <c r="I26" s="37"/>
+      <c r="J26" s="37"/>
+    </row>
+    <row r="27" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B27" s="37" t="s">
+        <v>56</v>
+      </c>
+      <c r="C27" s="37"/>
+      <c r="D27" s="37"/>
+      <c r="E27" s="37"/>
+      <c r="F27" s="37"/>
+      <c r="G27" s="37"/>
+      <c r="H27" s="37"/>
+      <c r="I27" s="37"/>
+      <c r="J27" s="37"/>
+    </row>
+    <row r="28" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B28" s="37" t="s">
+        <v>57</v>
+      </c>
+      <c r="C28" s="37"/>
+      <c r="D28" s="37"/>
+      <c r="E28" s="37"/>
+      <c r="F28" s="37"/>
+      <c r="G28" s="37"/>
+      <c r="H28" s="37"/>
+      <c r="I28" s="37"/>
+      <c r="J28" s="37"/>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="B2:J2"/>
+    <mergeCell ref="E16:J16"/>
+    <mergeCell ref="B24:J24"/>
+    <mergeCell ref="B25:J25"/>
+    <mergeCell ref="B26:J26"/>
+    <mergeCell ref="B27:J27"/>
+    <mergeCell ref="B28:J28"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B2:C13"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="75"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="75"/>
   </cols>
   <sheetData>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="24" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B4" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="C4" s="14" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="25" t="s">
-        <v>29</v>
-      </c>
-      <c r="C5" s="14" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="25" t="s">
-        <v>31</v>
-      </c>
-      <c r="C6" s="14" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="25" t="s">
-        <v>33</v>
-      </c>
-      <c r="C7" s="14" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="25" t="s">
-        <v>35</v>
-      </c>
-      <c r="C8" s="14" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="25" t="s">
-        <v>37</v>
-      </c>
-      <c r="C9" s="14" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="25" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B2" s="38" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B4" s="26" t="s">
+        <v>59</v>
+      </c>
+      <c r="C4" s="15" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B5" s="26" t="s">
+        <v>61</v>
+      </c>
+      <c r="C5" s="15" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B6" s="26" t="s">
         <v>39</v>
       </c>
-      <c r="C10" s="14" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="25" t="s">
-        <v>41</v>
-      </c>
-      <c r="C11" s="14" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="25" t="s">
-        <v>43</v>
-      </c>
-      <c r="C12" s="14" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="25" t="s">
-        <v>45</v>
-      </c>
-      <c r="C13" s="14" t="s">
-        <v>46</v>
+      <c r="C6" s="15" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B7" s="26" t="s">
+        <v>64</v>
+      </c>
+      <c r="C7" s="15" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B8" s="26" t="s">
+        <v>66</v>
+      </c>
+      <c r="C8" s="15" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B9" s="26" t="s">
+        <v>68</v>
+      </c>
+      <c r="C9" s="15" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B10" s="26" t="s">
+        <v>70</v>
+      </c>
+      <c r="C10" s="15" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B11" s="26" t="s">
+        <v>72</v>
+      </c>
+      <c r="C11" s="15" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B12" s="26" t="s">
+        <v>74</v>
+      </c>
+      <c r="C12" s="15" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B13" s="26" t="s">
+        <v>76</v>
+      </c>
+      <c r="C13" s="15" t="s">
+        <v>77</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Move trip gen table to standalone sheet; trim memo to threshold finding
Workbook restructured to TripGen (table only, formulas referencing a new
Rates sheet), Rates (ITE 12th Edition inputs + Durham UDO 3.3 threshold
check), AADT (growth projections, unchanged), and Dev. Memo drops the
Background Traffic Volumes section since the TIA determination rests
solely on site trips vs the 150-trip threshold; the conclusion keeps a
one-line reference to existing Page Road volumes (11,000 vpd, 2023 NCDOT
AADT) matching the template's style.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017bgXFHUDEAABZN3aMvsVWj
</commit_message>
<xml_diff>
--- a/3905_Page_Rd_Trip_Generation/Trip_Generation_3905_Page_Rd_Durham_NC.xlsx
+++ b/3905_Page_Rd_Trip_Generation/Trip_Generation_3905_Page_Rd_Durham_NC.xlsx
@@ -9,12 +9,13 @@
   </bookViews>
   <sheets>
     <sheet name="TripGen" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="AADT" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="Dev" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Rates" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="AADT" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Dev" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Area" vbProcedure="false">AADT!$B$2:$J$28</definedName>
-    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">TripGen!$B$2:$K$24</definedName>
+    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm.Print_Area" vbProcedure="false">AADT!$B$2:$J$28</definedName>
+    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">TripGen!$B$2:$K$11</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -91,7 +92,7 @@
     <t xml:space="preserve">Weekday (ADT)</t>
   </si>
   <si>
-    <t xml:space="preserve">Source: ITE Trip Generation Manual, 12th Edition. Blue cells are inputs.</t>
+    <t xml:space="preserve">Source: ITE Trip Generation Manual, 12th Edition. Blue cells are inputs; the TripGen table calculates from these rates.</t>
   </si>
   <si>
     <t xml:space="preserve">City of Durham TIA Threshold Check (UDO Section 3.3)</t>
@@ -465,15 +466,11 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="35">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -530,7 +527,7 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -550,7 +547,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -558,16 +555,12 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="11" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="11" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="169" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
@@ -590,20 +583,12 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="11" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="171" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="171" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="166" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -618,7 +603,7 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -814,278 +799,152 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="B1:K29"/>
+  <dimension ref="B1:K11"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="2.52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="9.52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="39.79"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="7.79"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="6" style="1" width="7.89"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="9.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="39.79"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="7.79"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="6" style="0" width="7.89"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="2" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
-      <c r="K2" s="2"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1"/>
+      <c r="J2" s="1"/>
+      <c r="K2" s="1"/>
     </row>
     <row r="3" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="4" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="F4" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G4" s="5"/>
-      <c r="H4" s="5"/>
-      <c r="I4" s="6" t="s">
+      <c r="G4" s="4"/>
+      <c r="H4" s="4"/>
+      <c r="I4" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="J4" s="6"/>
-      <c r="K4" s="6"/>
+      <c r="J4" s="5"/>
+      <c r="K4" s="5"/>
     </row>
     <row r="5" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B5" s="3"/>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
-      <c r="E5" s="4"/>
-      <c r="F5" s="7" t="s">
+      <c r="B5" s="2"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="G5" s="7" t="s">
+      <c r="G5" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="H5" s="7" t="s">
+      <c r="H5" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="I5" s="7" t="s">
+      <c r="I5" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="J5" s="7" t="s">
+      <c r="J5" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="K5" s="8" t="s">
+      <c r="K5" s="7" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B6" s="9" t="s">
+      <c r="B6" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="9"/>
-      <c r="D6" s="9"/>
-      <c r="E6" s="9"/>
-      <c r="F6" s="9"/>
-      <c r="G6" s="9"/>
-      <c r="H6" s="9"/>
-      <c r="I6" s="9"/>
-      <c r="J6" s="9"/>
-      <c r="K6" s="9"/>
+      <c r="C6" s="8"/>
+      <c r="D6" s="8"/>
+      <c r="E6" s="8"/>
+      <c r="F6" s="8"/>
+      <c r="G6" s="8"/>
+      <c r="H6" s="8"/>
+      <c r="I6" s="8"/>
+      <c r="J6" s="8"/>
+      <c r="K6" s="8"/>
     </row>
     <row r="7" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B7" s="10" t="n">
+      <c r="B7" s="9" t="n">
         <v>110</v>
       </c>
-      <c r="C7" s="11" t="s">
+      <c r="C7" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="D7" s="12" t="n">
+      <c r="D7" s="11" t="n">
         <v>150000</v>
       </c>
-      <c r="E7" s="13" t="n">
-        <f aca="false">IF(D7&gt;0,ROUND($D$16*(D7/1000),0),0)</f>
+      <c r="E7" s="12" t="n">
+        <f aca="false">IF(D7&gt;0,ROUND(Rates!$D$5*(D7/1000),0),0)</f>
         <v>540</v>
       </c>
-      <c r="F7" s="13" t="n">
-        <f aca="false">IF(D7&gt;0,ROUND($E$17*H7,0),0)</f>
+      <c r="F7" s="12" t="n">
+        <f aca="false">IF(D7&gt;0,ROUND(Rates!$E$6*H7,0),0)</f>
         <v>62</v>
       </c>
-      <c r="G7" s="13" t="n">
+      <c r="G7" s="12" t="n">
         <f aca="false">H7-F7</f>
         <v>10</v>
       </c>
-      <c r="H7" s="13" t="n">
-        <f aca="false">IF(D7&gt;0,ROUND($D$17*(D7/1000),0),0)</f>
+      <c r="H7" s="12" t="n">
+        <f aca="false">IF(D7&gt;0,ROUND(Rates!$D$6*(D7/1000),0),0)</f>
         <v>72</v>
       </c>
-      <c r="I7" s="13" t="n">
-        <f aca="false">IF(D7&gt;0,ROUND($E$18*K7,0),0)</f>
+      <c r="I7" s="12" t="n">
+        <f aca="false">IF(D7&gt;0,ROUND(Rates!$E$7*K7,0),0)</f>
         <v>18</v>
       </c>
-      <c r="J7" s="13" t="n">
+      <c r="J7" s="12" t="n">
         <f aca="false">K7-I7</f>
         <v>56</v>
       </c>
-      <c r="K7" s="14" t="n">
-        <f aca="false">IF(D7&gt;0,ROUND($D$18*(D7/1000),0),0)</f>
+      <c r="K7" s="13" t="n">
+        <f aca="false">IF(D7&gt;0,ROUND(Rates!$D$7*(D7/1000),0),0)</f>
         <v>74</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="9" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B9" s="15" t="s">
+      <c r="B9" s="14" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B10" s="15" t="s">
+      <c r="B10" s="14" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B11" s="15" t="s">
+      <c r="B11" s="14" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="13" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="14" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B14" s="16" t="s">
-        <v>15</v>
-      </c>
-      <c r="C14" s="16"/>
-      <c r="D14" s="16"/>
-      <c r="E14" s="16"/>
-      <c r="F14" s="16"/>
-    </row>
-    <row r="15" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B15" s="17" t="s">
-        <v>16</v>
-      </c>
-      <c r="C15" s="17"/>
-      <c r="D15" s="17" t="s">
-        <v>17</v>
-      </c>
-      <c r="E15" s="17" t="s">
-        <v>18</v>
-      </c>
-      <c r="F15" s="17" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B16" s="18" t="s">
-        <v>20</v>
-      </c>
-      <c r="C16" s="18"/>
-      <c r="D16" s="19" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="E16" s="20" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="F16" s="20" t="n">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B17" s="18" t="s">
-        <v>5</v>
-      </c>
-      <c r="C17" s="18"/>
-      <c r="D17" s="19" t="n">
-        <v>0.48</v>
-      </c>
-      <c r="E17" s="20" t="n">
-        <v>0.86</v>
-      </c>
-      <c r="F17" s="20" t="n">
-        <v>0.14</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B18" s="18" t="s">
-        <v>6</v>
-      </c>
-      <c r="C18" s="18"/>
-      <c r="D18" s="19" t="n">
-        <v>0.49</v>
-      </c>
-      <c r="E18" s="20" t="n">
-        <v>0.24</v>
-      </c>
-      <c r="F18" s="20" t="n">
-        <v>0.76</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B19" s="21" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="21" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B21" s="16" t="s">
-        <v>22</v>
-      </c>
-      <c r="C21" s="16"/>
-      <c r="D21" s="16"/>
-      <c r="E21" s="16"/>
-      <c r="F21" s="16"/>
-    </row>
-    <row r="22" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B22" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="C22" s="18"/>
-      <c r="D22" s="22" t="n">
-        <v>150</v>
-      </c>
-      <c r="E22" s="23"/>
-      <c r="F22" s="23"/>
-    </row>
-    <row r="23" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B23" s="18" t="s">
-        <v>24</v>
-      </c>
-      <c r="C23" s="18"/>
-      <c r="D23" s="24" t="n">
-        <f aca="false">MAX(H7,K7)</f>
-        <v>74</v>
-      </c>
-      <c r="E23" s="23"/>
-      <c r="F23" s="23"/>
-    </row>
-    <row r="24" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B24" s="18" t="s">
-        <v>25</v>
-      </c>
-      <c r="C24" s="18"/>
-      <c r="D24" s="17" t="str">
-        <f aca="false">IF(AND(H7&lt;D22,K7&lt;D22),"TIA Not Required","TIA Required")</f>
-        <v>TIA Not Required</v>
-      </c>
-      <c r="E24" s="17"/>
-      <c r="F24" s="17"/>
-    </row>
-    <row r="25" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="26" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="27" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="28" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="29" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <mergeCells count="18">
+  <mergeCells count="8">
     <mergeCell ref="B2:K2"/>
     <mergeCell ref="B4:B5"/>
     <mergeCell ref="C4:C5"/>
@@ -1094,16 +953,6 @@
     <mergeCell ref="F4:H4"/>
     <mergeCell ref="I4:K4"/>
     <mergeCell ref="B6:K6"/>
-    <mergeCell ref="B14:F14"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="B21:F21"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="D24:F24"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1118,6 +967,170 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="B2:G14"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="4" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="30"/>
+  </cols>
+  <sheetData>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B2" s="15" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="15"/>
+      <c r="G2" s="15"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B4" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" s="16"/>
+      <c r="D4" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="E4" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="F4" s="16" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B5" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" s="17"/>
+      <c r="D5" s="18" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="E5" s="19" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F5" s="19" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B6" s="17" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" s="17"/>
+      <c r="D6" s="18" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="E6" s="19" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="F6" s="19" t="n">
+        <v>0.14</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B7" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="C7" s="17"/>
+      <c r="D7" s="18" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="E7" s="19" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="F7" s="19" t="n">
+        <v>0.76</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B8" s="20" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" s="20"/>
+      <c r="D8" s="20"/>
+      <c r="E8" s="20"/>
+      <c r="F8" s="20"/>
+      <c r="G8" s="20"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B11" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="C11" s="15"/>
+      <c r="D11" s="15"/>
+      <c r="E11" s="15"/>
+      <c r="F11" s="15"/>
+      <c r="G11" s="15"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B12" s="17" t="s">
+        <v>23</v>
+      </c>
+      <c r="C12" s="17"/>
+      <c r="D12" s="21" t="n">
+        <v>150</v>
+      </c>
+      <c r="E12" s="22"/>
+      <c r="F12" s="22"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B13" s="17" t="s">
+        <v>24</v>
+      </c>
+      <c r="C13" s="17"/>
+      <c r="D13" s="23" t="n">
+        <f aca="false">MAX(TripGen!H7,TripGen!K7)</f>
+        <v>74</v>
+      </c>
+      <c r="E13" s="22"/>
+      <c r="F13" s="22"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B14" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="C14" s="17"/>
+      <c r="D14" s="16" t="str">
+        <f aca="false">IF(AND(TripGen!H7&lt;D12,TripGen!K7&lt;D12),"TIA Not Required","TIA Required")</f>
+        <v>TIA Not Required</v>
+      </c>
+      <c r="E14" s="16"/>
+      <c r="F14" s="16"/>
+    </row>
+  </sheetData>
+  <mergeCells count="11">
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B8:G8"/>
+    <mergeCell ref="B11:G11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="D14:F14"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="B2:J28"/>
@@ -1130,292 +1143,292 @@
   </cols>
   <sheetData>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="25" t="s">
+      <c r="B2" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
-      <c r="F2" s="25"/>
-      <c r="G2" s="25"/>
-      <c r="H2" s="25"/>
-      <c r="I2" s="25"/>
-      <c r="J2" s="25"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="15"/>
+      <c r="G2" s="15"/>
+      <c r="H2" s="15"/>
+      <c r="I2" s="15"/>
+      <c r="J2" s="15"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B4" s="26" t="s">
+      <c r="B4" s="24" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="17" t="s">
+      <c r="B5" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="C5" s="17" t="s">
+      <c r="C5" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="D5" s="17" t="s">
+      <c r="D5" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="E5" s="17" t="s">
+      <c r="E5" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="F5" s="17" t="s">
+      <c r="F5" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="G5" s="17" t="s">
+      <c r="G5" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="H5" s="17" t="s">
+      <c r="H5" s="16" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="18" t="s">
+      <c r="B6" s="17" t="s">
         <v>35</v>
       </c>
-      <c r="C6" s="27" t="n">
+      <c r="C6" s="25" t="n">
         <v>6700</v>
       </c>
-      <c r="D6" s="27" t="n">
+      <c r="D6" s="25" t="n">
         <v>7700</v>
       </c>
-      <c r="E6" s="27" t="n">
+      <c r="E6" s="25" t="n">
         <v>9900</v>
       </c>
-      <c r="F6" s="24" t="s">
+      <c r="F6" s="23" t="s">
         <v>36</v>
       </c>
-      <c r="G6" s="27" t="n">
+      <c r="G6" s="25" t="n">
         <v>10000</v>
       </c>
-      <c r="H6" s="27" t="n">
+      <c r="H6" s="25" t="n">
         <v>11000</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="18" t="s">
+      <c r="B7" s="17" t="s">
         <v>37</v>
       </c>
-      <c r="C7" s="27" t="n">
+      <c r="C7" s="25" t="n">
         <v>8000</v>
       </c>
-      <c r="D7" s="27" t="n">
+      <c r="D7" s="25" t="n">
         <v>5500</v>
       </c>
-      <c r="E7" s="27" t="n">
+      <c r="E7" s="25" t="n">
         <v>6800</v>
       </c>
-      <c r="F7" s="27" t="n">
+      <c r="F7" s="25" t="n">
         <v>8200</v>
       </c>
-      <c r="G7" s="27" t="n">
+      <c r="G7" s="25" t="n">
         <v>6600</v>
       </c>
-      <c r="H7" s="27" t="n">
+      <c r="H7" s="25" t="n">
         <v>7100</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="26" t="s">
+      <c r="B10" s="24" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="17" t="s">
+      <c r="B11" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="C11" s="17" t="s">
+      <c r="C11" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="D11" s="17" t="s">
+      <c r="D11" s="16" t="s">
         <v>41</v>
       </c>
-      <c r="E11" s="17" t="s">
+      <c r="E11" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="F11" s="17" t="s">
+      <c r="F11" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="G11" s="17" t="s">
+      <c r="G11" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="H11" s="17" t="s">
+      <c r="H11" s="16" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="18" t="s">
+      <c r="B12" s="17" t="s">
         <v>46</v>
       </c>
-      <c r="C12" s="28" t="n">
+      <c r="C12" s="26" t="n">
         <f aca="false">H6</f>
         <v>11000</v>
       </c>
-      <c r="D12" s="29" t="n">
+      <c r="D12" s="27" t="n">
         <f aca="false">(H6/C6)^(1/10)-1</f>
         <v>0.050828367580992</v>
       </c>
-      <c r="E12" s="29" t="n">
+      <c r="E12" s="27" t="n">
         <f aca="false">(H6/E6)^(1/6)-1</f>
         <v>0.0177151706893666</v>
       </c>
-      <c r="F12" s="30" t="n">
+      <c r="F12" s="28" t="n">
         <v>0.03</v>
       </c>
-      <c r="G12" s="28" t="n">
+      <c r="G12" s="26" t="n">
         <f aca="false">C12*(1+F12)^($D$16-2023)</f>
         <v>12752.0148173</v>
       </c>
-      <c r="H12" s="28" t="n">
+      <c r="H12" s="26" t="n">
         <f aca="false">ROUND(G12,-2)</f>
         <v>12800</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="18" t="s">
+      <c r="B13" s="17" t="s">
         <v>47</v>
       </c>
-      <c r="C13" s="28" t="n">
+      <c r="C13" s="26" t="n">
         <f aca="false">H7</f>
         <v>7100</v>
       </c>
-      <c r="D13" s="29" t="n">
+      <c r="D13" s="27" t="n">
         <f aca="false">(H7/C7)^(1/10)-1</f>
         <v>-0.0118637399993557</v>
       </c>
-      <c r="E13" s="29" t="n">
+      <c r="E13" s="27" t="n">
         <f aca="false">(H7/E7)^(1/6)-1</f>
         <v>0.0072213107942356</v>
       </c>
-      <c r="F13" s="30" t="n">
+      <c r="F13" s="28" t="n">
         <v>0.03</v>
       </c>
-      <c r="G13" s="28" t="n">
+      <c r="G13" s="26" t="n">
         <f aca="false">C13*(1+F13)^($D$16-2023)</f>
         <v>8230.84592753</v>
       </c>
-      <c r="H13" s="28" t="n">
+      <c r="H13" s="26" t="n">
         <f aca="false">ROUND(G13,-2)</f>
         <v>8200</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="18" t="s">
+      <c r="B15" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="C15" s="31"/>
-      <c r="D15" s="32" t="n">
+      <c r="C15" s="22"/>
+      <c r="D15" s="29" t="n">
         <v>2027</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="18" t="s">
+      <c r="B16" s="17" t="s">
         <v>49</v>
       </c>
-      <c r="C16" s="31"/>
-      <c r="D16" s="33" t="n">
+      <c r="C16" s="22"/>
+      <c r="D16" s="30" t="n">
         <f aca="false">D15+1</f>
         <v>2028</v>
       </c>
-      <c r="E16" s="34" t="s">
+      <c r="E16" s="20" t="s">
         <v>50</v>
       </c>
-      <c r="F16" s="34"/>
-      <c r="G16" s="34"/>
-      <c r="H16" s="34"/>
-      <c r="I16" s="34"/>
-      <c r="J16" s="34"/>
+      <c r="F16" s="20"/>
+      <c r="G16" s="20"/>
+      <c r="H16" s="20"/>
+      <c r="I16" s="20"/>
+      <c r="J16" s="20"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="26" t="s">
+      <c r="B19" s="24" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="18" t="s">
+      <c r="B20" s="17" t="s">
         <v>52</v>
       </c>
-      <c r="C20" s="31"/>
-      <c r="D20" s="35" t="n">
+      <c r="C20" s="22"/>
+      <c r="D20" s="31" t="n">
         <f aca="false">C12-C13</f>
         <v>3900</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="18" t="s">
+      <c r="B21" s="17" t="s">
         <v>53</v>
       </c>
-      <c r="C21" s="31"/>
-      <c r="D21" s="36" t="n">
+      <c r="C21" s="22"/>
+      <c r="D21" s="32" t="n">
         <f aca="false">ROUND(D20*(1+F12)^($D$16-2023),-2)</f>
         <v>4500</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B24" s="37" t="s">
+      <c r="B24" s="33" t="s">
         <v>12</v>
       </c>
-      <c r="C24" s="37"/>
-      <c r="D24" s="37"/>
-      <c r="E24" s="37"/>
-      <c r="F24" s="37"/>
-      <c r="G24" s="37"/>
-      <c r="H24" s="37"/>
-      <c r="I24" s="37"/>
-      <c r="J24" s="37"/>
+      <c r="C24" s="33"/>
+      <c r="D24" s="33"/>
+      <c r="E24" s="33"/>
+      <c r="F24" s="33"/>
+      <c r="G24" s="33"/>
+      <c r="H24" s="33"/>
+      <c r="I24" s="33"/>
+      <c r="J24" s="33"/>
     </row>
     <row r="25" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B25" s="37" t="s">
+      <c r="B25" s="33" t="s">
         <v>54</v>
       </c>
-      <c r="C25" s="37"/>
-      <c r="D25" s="37"/>
-      <c r="E25" s="37"/>
-      <c r="F25" s="37"/>
-      <c r="G25" s="37"/>
-      <c r="H25" s="37"/>
-      <c r="I25" s="37"/>
-      <c r="J25" s="37"/>
+      <c r="C25" s="33"/>
+      <c r="D25" s="33"/>
+      <c r="E25" s="33"/>
+      <c r="F25" s="33"/>
+      <c r="G25" s="33"/>
+      <c r="H25" s="33"/>
+      <c r="I25" s="33"/>
+      <c r="J25" s="33"/>
     </row>
     <row r="26" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B26" s="37" t="s">
+      <c r="B26" s="33" t="s">
         <v>55</v>
       </c>
-      <c r="C26" s="37"/>
-      <c r="D26" s="37"/>
-      <c r="E26" s="37"/>
-      <c r="F26" s="37"/>
-      <c r="G26" s="37"/>
-      <c r="H26" s="37"/>
-      <c r="I26" s="37"/>
-      <c r="J26" s="37"/>
+      <c r="C26" s="33"/>
+      <c r="D26" s="33"/>
+      <c r="E26" s="33"/>
+      <c r="F26" s="33"/>
+      <c r="G26" s="33"/>
+      <c r="H26" s="33"/>
+      <c r="I26" s="33"/>
+      <c r="J26" s="33"/>
     </row>
     <row r="27" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B27" s="37" t="s">
+      <c r="B27" s="33" t="s">
         <v>56</v>
       </c>
-      <c r="C27" s="37"/>
-      <c r="D27" s="37"/>
-      <c r="E27" s="37"/>
-      <c r="F27" s="37"/>
-      <c r="G27" s="37"/>
-      <c r="H27" s="37"/>
-      <c r="I27" s="37"/>
-      <c r="J27" s="37"/>
+      <c r="C27" s="33"/>
+      <c r="D27" s="33"/>
+      <c r="E27" s="33"/>
+      <c r="F27" s="33"/>
+      <c r="G27" s="33"/>
+      <c r="H27" s="33"/>
+      <c r="I27" s="33"/>
+      <c r="J27" s="33"/>
     </row>
     <row r="28" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B28" s="37" t="s">
+      <c r="B28" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="C28" s="37"/>
-      <c r="D28" s="37"/>
-      <c r="E28" s="37"/>
-      <c r="F28" s="37"/>
-      <c r="G28" s="37"/>
-      <c r="H28" s="37"/>
-      <c r="I28" s="37"/>
-      <c r="J28" s="37"/>
+      <c r="C28" s="33"/>
+      <c r="D28" s="33"/>
+      <c r="E28" s="33"/>
+      <c r="F28" s="33"/>
+      <c r="G28" s="33"/>
+      <c r="H28" s="33"/>
+      <c r="I28" s="33"/>
+      <c r="J28" s="33"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -1437,7 +1450,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -1445,92 +1458,92 @@
   <dimension ref="B2:C13"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="75"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="75"/>
   </cols>
   <sheetData>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B2" s="38" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B2" s="34" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B4" s="26" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B4" s="24" t="s">
         <v>59</v>
       </c>
-      <c r="C4" s="15" t="s">
+      <c r="C4" s="14" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B5" s="26" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B5" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="C5" s="15" t="s">
+      <c r="C5" s="14" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B6" s="26" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B6" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="C6" s="15" t="s">
+      <c r="C6" s="14" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B7" s="26" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B7" s="24" t="s">
         <v>64</v>
       </c>
-      <c r="C7" s="15" t="s">
+      <c r="C7" s="14" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B8" s="26" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B8" s="24" t="s">
         <v>66</v>
       </c>
-      <c r="C8" s="15" t="s">
+      <c r="C8" s="14" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B9" s="26" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B9" s="24" t="s">
         <v>68</v>
       </c>
-      <c r="C9" s="15" t="s">
+      <c r="C9" s="14" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B10" s="26" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B10" s="24" t="s">
         <v>70</v>
       </c>
-      <c r="C10" s="15" t="s">
+      <c r="C10" s="14" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B11" s="26" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B11" s="24" t="s">
         <v>72</v>
       </c>
-      <c r="C11" s="15" t="s">
+      <c r="C11" s="14" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B12" s="26" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B12" s="24" t="s">
         <v>74</v>
       </c>
-      <c r="C12" s="15" t="s">
+      <c r="C12" s="14" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B13" s="26" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B13" s="24" t="s">
         <v>76</v>
       </c>
-      <c r="C13" s="15" t="s">
+      <c r="C13" s="14" t="s">
         <v>77</v>
       </c>
     </row>

</xml_diff>

<commit_message>
End NCDOT sentence at threshold; correct 2023 AADT to station value
Memo: the NCDOT sentence now ends at "well below the NCDOT TIA
threshold of 3,000 daily trips" without speculating on the driveway
permit outcome. Workbook AADT sheet: Page Rd south of Airport Rd 2023
AADT corrected from the segment-layer value (11,000) to the fully
scrolled station history value (8,800, station 0320000269); the
discrepancy is documented in the notes. Recomputed south-leg CAGRs
(2.8% / -1.9%), 2028 Build volume (10,200 vpd), and Airport Rd
difference floor (1,700 vpd).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017bgXFHUDEAABZN3aMvsVWj
</commit_message>
<xml_diff>
--- a/3905_Page_Rd_Trip_Generation/Trip_Generation_3905_Page_Rd_Durham_NC.xlsx
+++ b/3905_Page_Rd_Trip_Generation/Trip_Generation_3905_Page_Rd_Durham_NC.xlsx
@@ -191,10 +191,10 @@
     <t xml:space="preserve">Projected to Build year at selected rate (south leg)</t>
   </si>
   <si>
-    <t xml:space="preserve">1. 2023 values are from the NCDOT AADT traffic segment layer (Route 40001973032 = SR 1973/Page Rd; segments MP 3.334-3.620 [TMS 0320000269, AADT 11,000] and MP 2.728-3.334 [TMS 0320000260, AADT 7,100], source "Maintenance"). Earlier years are from the NCDOT AADT station history (ncdot.maps.arcgis.com), retrieved August 2026.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2. Selected growth rate is an engineering input (blue). Computed CAGRs bracket it: south leg 5.1% (2013-2023) / 1.8% (2017-2023); north leg -1.2% (2013-2023) / 0.7% (2017-2023). 3.0%/yr compounded is applied corridor-wide as a conservative planning rate.</t>
+    <t xml:space="preserve">1. AADT history from the NCDOT AADT station layer (ncdot.maps.arcgis.com, retrieved August 2026): stations 0320000269 (Page Rd south of Airport Rd) and 0320000260 (Page Rd north of Airport Rd). Note: the NCDOT AADT traffic segment layer (Route 40001973032, MP 3.334-3.620, source "Maintenance") displays 11,000 vpd for the segment south of Airport Rd versus the 8,800 station history value; the published station count history is used here. The north segment (MP 2.728-3.334) matches its station history (7,100 vpd).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. Selected growth rate is an engineering input (blue). Computed CAGRs bracket it: south leg 2.8% (2013-2023) / -1.9% (2017-2023); north leg -1.2% (2013-2023) / 0.7% (2017-2023). 3.0%/yr compounded is applied corridor-wide as a conservative planning rate above the observed long-term trend at both stations.</t>
   </si>
   <si>
     <t xml:space="preserve">3. Build AADT = 2023 AADT x (1 + selected rate)^(Build year - 2023). Build year per City of Durham TIA Guidelines (durhamnc.gov, "Guidelines for Traffic Impact Analysis (TIA) Requirement"): the analysis must examine expected traffic conditions one year after the project is scheduled to be complete; with an assumed 2027 opening, Build year = 2028.</t>
@@ -466,11 +466,15 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="36">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -555,7 +559,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="11" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="11" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -603,7 +607,7 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -802,144 +806,144 @@
   <dimension ref="B1:K11"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2.52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="9.52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="39.79"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="7.79"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="6" style="0" width="7.89"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="2.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="9.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="39.79"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="7.79"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="6" style="1" width="7.89"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="2" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1"/>
-      <c r="J2" s="1"/>
-      <c r="K2" s="1"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
+      <c r="J2" s="2"/>
+      <c r="K2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="4" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="F4" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="G4" s="4"/>
-      <c r="H4" s="4"/>
-      <c r="I4" s="5" t="s">
+      <c r="G4" s="5"/>
+      <c r="H4" s="5"/>
+      <c r="I4" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="J4" s="5"/>
-      <c r="K4" s="5"/>
+      <c r="J4" s="6"/>
+      <c r="K4" s="6"/>
     </row>
     <row r="5" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B5" s="2"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="6" t="s">
+      <c r="B5" s="3"/>
+      <c r="C5" s="4"/>
+      <c r="D5" s="4"/>
+      <c r="E5" s="4"/>
+      <c r="F5" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="G5" s="6" t="s">
+      <c r="G5" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="H5" s="6" t="s">
+      <c r="H5" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="I5" s="6" t="s">
+      <c r="I5" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="J5" s="6" t="s">
+      <c r="J5" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="K5" s="7" t="s">
+      <c r="K5" s="8" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B6" s="8" t="s">
+      <c r="B6" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="8"/>
-      <c r="D6" s="8"/>
-      <c r="E6" s="8"/>
-      <c r="F6" s="8"/>
-      <c r="G6" s="8"/>
-      <c r="H6" s="8"/>
-      <c r="I6" s="8"/>
-      <c r="J6" s="8"/>
-      <c r="K6" s="8"/>
+      <c r="C6" s="9"/>
+      <c r="D6" s="9"/>
+      <c r="E6" s="9"/>
+      <c r="F6" s="9"/>
+      <c r="G6" s="9"/>
+      <c r="H6" s="9"/>
+      <c r="I6" s="9"/>
+      <c r="J6" s="9"/>
+      <c r="K6" s="9"/>
     </row>
     <row r="7" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B7" s="9" t="n">
+      <c r="B7" s="10" t="n">
         <v>110</v>
       </c>
-      <c r="C7" s="10" t="s">
+      <c r="C7" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="D7" s="11" t="n">
+      <c r="D7" s="12" t="n">
         <v>150000</v>
       </c>
-      <c r="E7" s="12" t="n">
+      <c r="E7" s="13" t="n">
         <f aca="false">IF(D7&gt;0,ROUND(Rates!$D$5*(D7/1000),0),0)</f>
         <v>540</v>
       </c>
-      <c r="F7" s="12" t="n">
+      <c r="F7" s="13" t="n">
         <f aca="false">IF(D7&gt;0,ROUND(Rates!$E$6*H7,0),0)</f>
         <v>62</v>
       </c>
-      <c r="G7" s="12" t="n">
+      <c r="G7" s="13" t="n">
         <f aca="false">H7-F7</f>
         <v>10</v>
       </c>
-      <c r="H7" s="12" t="n">
+      <c r="H7" s="13" t="n">
         <f aca="false">IF(D7&gt;0,ROUND(Rates!$D$6*(D7/1000),0),0)</f>
         <v>72</v>
       </c>
-      <c r="I7" s="12" t="n">
+      <c r="I7" s="13" t="n">
         <f aca="false">IF(D7&gt;0,ROUND(Rates!$E$7*K7,0),0)</f>
         <v>18</v>
       </c>
-      <c r="J7" s="12" t="n">
+      <c r="J7" s="13" t="n">
         <f aca="false">K7-I7</f>
         <v>56</v>
       </c>
-      <c r="K7" s="13" t="n">
+      <c r="K7" s="14" t="n">
         <f aca="false">IF(D7&gt;0,ROUND(Rates!$D$7*(D7/1000),0),0)</f>
         <v>74</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="9" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B9" s="14" t="s">
+      <c r="B9" s="15" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B10" s="14" t="s">
+      <c r="B10" s="15" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B11" s="14" t="s">
+      <c r="B11" s="15" t="s">
         <v>14</v>
       </c>
     </row>
@@ -972,137 +976,137 @@
   <dimension ref="B2:G14"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="4" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="2.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="4" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="30"/>
   </cols>
   <sheetData>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="15" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B2" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="15"/>
-      <c r="D2" s="15"/>
-      <c r="E2" s="15"/>
-      <c r="F2" s="15"/>
-      <c r="G2" s="15"/>
+      <c r="C2" s="16"/>
+      <c r="D2" s="16"/>
+      <c r="E2" s="16"/>
+      <c r="F2" s="16"/>
+      <c r="G2" s="16"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B4" s="16" t="s">
+      <c r="B4" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="16"/>
-      <c r="D4" s="16" t="s">
+      <c r="C4" s="17"/>
+      <c r="D4" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="E4" s="16" t="s">
+      <c r="E4" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="F4" s="16" t="s">
+      <c r="F4" s="17" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="17" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B5" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="C5" s="17"/>
-      <c r="D5" s="18" t="n">
+      <c r="C5" s="18"/>
+      <c r="D5" s="19" t="n">
         <v>3.6</v>
       </c>
-      <c r="E5" s="19" t="n">
+      <c r="E5" s="20" t="n">
         <v>0.5</v>
       </c>
-      <c r="F5" s="19" t="n">
+      <c r="F5" s="20" t="n">
         <v>0.5</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="17" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B6" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="17"/>
-      <c r="D6" s="18" t="n">
+      <c r="C6" s="18"/>
+      <c r="D6" s="19" t="n">
         <v>0.48</v>
       </c>
-      <c r="E6" s="19" t="n">
+      <c r="E6" s="20" t="n">
         <v>0.86</v>
       </c>
-      <c r="F6" s="19" t="n">
+      <c r="F6" s="20" t="n">
         <v>0.14</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="17" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B7" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="17"/>
-      <c r="D7" s="18" t="n">
+      <c r="C7" s="18"/>
+      <c r="D7" s="19" t="n">
         <v>0.49</v>
       </c>
-      <c r="E7" s="19" t="n">
+      <c r="E7" s="20" t="n">
         <v>0.24</v>
       </c>
-      <c r="F7" s="19" t="n">
+      <c r="F7" s="20" t="n">
         <v>0.76</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="20" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B8" s="21" t="s">
         <v>21</v>
       </c>
-      <c r="C8" s="20"/>
-      <c r="D8" s="20"/>
-      <c r="E8" s="20"/>
-      <c r="F8" s="20"/>
-      <c r="G8" s="20"/>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="15" t="s">
+      <c r="C8" s="21"/>
+      <c r="D8" s="21"/>
+      <c r="E8" s="21"/>
+      <c r="F8" s="21"/>
+      <c r="G8" s="21"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B11" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="C11" s="15"/>
-      <c r="D11" s="15"/>
-      <c r="E11" s="15"/>
-      <c r="F11" s="15"/>
-      <c r="G11" s="15"/>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="17" t="s">
+      <c r="C11" s="16"/>
+      <c r="D11" s="16"/>
+      <c r="E11" s="16"/>
+      <c r="F11" s="16"/>
+      <c r="G11" s="16"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B12" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="C12" s="17"/>
-      <c r="D12" s="21" t="n">
+      <c r="C12" s="18"/>
+      <c r="D12" s="22" t="n">
         <v>150</v>
       </c>
-      <c r="E12" s="22"/>
-      <c r="F12" s="22"/>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="17" t="s">
+      <c r="E12" s="23"/>
+      <c r="F12" s="23"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B13" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="C13" s="17"/>
-      <c r="D13" s="23" t="n">
+      <c r="C13" s="18"/>
+      <c r="D13" s="24" t="n">
         <f aca="false">MAX(TripGen!H7,TripGen!K7)</f>
         <v>74</v>
       </c>
-      <c r="E13" s="22"/>
-      <c r="F13" s="22"/>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="17" t="s">
+      <c r="E13" s="23"/>
+      <c r="F13" s="23"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B14" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="C14" s="17"/>
-      <c r="D14" s="16" t="str">
+      <c r="C14" s="18"/>
+      <c r="D14" s="17" t="str">
         <f aca="false">IF(AND(TripGen!H7&lt;D12,TripGen!K7&lt;D12),"TIA Not Required","TIA Required")</f>
         <v>TIA Not Required</v>
       </c>
-      <c r="E14" s="16"/>
-      <c r="F14" s="16"/>
+      <c r="E14" s="17"/>
+      <c r="F14" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="11">
@@ -1136,299 +1140,299 @@
   <dimension ref="B2:J28"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="3" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="2.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="3" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="1" width="13"/>
   </cols>
   <sheetData>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="15" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B2" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="C2" s="15"/>
-      <c r="D2" s="15"/>
-      <c r="E2" s="15"/>
-      <c r="F2" s="15"/>
-      <c r="G2" s="15"/>
-      <c r="H2" s="15"/>
-      <c r="I2" s="15"/>
-      <c r="J2" s="15"/>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B4" s="24" t="s">
+      <c r="C2" s="16"/>
+      <c r="D2" s="16"/>
+      <c r="E2" s="16"/>
+      <c r="F2" s="16"/>
+      <c r="G2" s="16"/>
+      <c r="H2" s="16"/>
+      <c r="I2" s="16"/>
+      <c r="J2" s="16"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B4" s="25" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="16" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B5" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="C5" s="16" t="s">
+      <c r="C5" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="D5" s="16" t="s">
+      <c r="D5" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="E5" s="16" t="s">
+      <c r="E5" s="17" t="s">
         <v>31</v>
       </c>
-      <c r="F5" s="16" t="s">
+      <c r="F5" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="G5" s="16" t="s">
+      <c r="G5" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="H5" s="16" t="s">
+      <c r="H5" s="17" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="17" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B6" s="18" t="s">
         <v>35</v>
       </c>
-      <c r="C6" s="25" t="n">
+      <c r="C6" s="26" t="n">
         <v>6700</v>
       </c>
-      <c r="D6" s="25" t="n">
+      <c r="D6" s="26" t="n">
         <v>7700</v>
       </c>
-      <c r="E6" s="25" t="n">
+      <c r="E6" s="26" t="n">
         <v>9900</v>
       </c>
-      <c r="F6" s="23" t="s">
+      <c r="F6" s="24" t="s">
         <v>36</v>
       </c>
-      <c r="G6" s="25" t="n">
+      <c r="G6" s="26" t="n">
         <v>10000</v>
       </c>
-      <c r="H6" s="25" t="n">
-        <v>11000</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="17" t="s">
+      <c r="H6" s="26" t="n">
+        <v>8800</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B7" s="18" t="s">
         <v>37</v>
       </c>
-      <c r="C7" s="25" t="n">
+      <c r="C7" s="26" t="n">
         <v>8000</v>
       </c>
-      <c r="D7" s="25" t="n">
+      <c r="D7" s="26" t="n">
         <v>5500</v>
       </c>
-      <c r="E7" s="25" t="n">
+      <c r="E7" s="26" t="n">
         <v>6800</v>
       </c>
-      <c r="F7" s="25" t="n">
+      <c r="F7" s="26" t="n">
         <v>8200</v>
       </c>
-      <c r="G7" s="25" t="n">
+      <c r="G7" s="26" t="n">
         <v>6600</v>
       </c>
-      <c r="H7" s="25" t="n">
+      <c r="H7" s="26" t="n">
         <v>7100</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="24" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B10" s="25" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="16" t="s">
+    <row r="11" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B11" s="17" t="s">
         <v>39</v>
       </c>
-      <c r="C11" s="16" t="s">
+      <c r="C11" s="17" t="s">
         <v>40</v>
       </c>
-      <c r="D11" s="16" t="s">
+      <c r="D11" s="17" t="s">
         <v>41</v>
       </c>
-      <c r="E11" s="16" t="s">
+      <c r="E11" s="17" t="s">
         <v>42</v>
       </c>
-      <c r="F11" s="16" t="s">
+      <c r="F11" s="17" t="s">
         <v>43</v>
       </c>
-      <c r="G11" s="16" t="s">
+      <c r="G11" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="H11" s="16" t="s">
+      <c r="H11" s="17" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="17" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B12" s="18" t="s">
         <v>46</v>
       </c>
-      <c r="C12" s="26" t="n">
+      <c r="C12" s="27" t="n">
         <f aca="false">H6</f>
-        <v>11000</v>
-      </c>
-      <c r="D12" s="27" t="n">
+        <v>8800</v>
+      </c>
+      <c r="D12" s="28" t="n">
         <f aca="false">(H6/C6)^(1/10)-1</f>
-        <v>0.050828367580992</v>
-      </c>
-      <c r="E12" s="27" t="n">
+        <v>0.0276394947719256</v>
+      </c>
+      <c r="E12" s="28" t="n">
         <f aca="false">(H6/E6)^(1/6)-1</f>
-        <v>0.0177151706893666</v>
-      </c>
-      <c r="F12" s="28" t="n">
+        <v>-0.01943908218904</v>
+      </c>
+      <c r="F12" s="29" t="n">
         <v>0.03</v>
       </c>
-      <c r="G12" s="26" t="n">
+      <c r="G12" s="27" t="n">
         <f aca="false">C12*(1+F12)^($D$16-2023)</f>
-        <v>12752.0148173</v>
-      </c>
-      <c r="H12" s="26" t="n">
+        <v>10201.61185384</v>
+      </c>
+      <c r="H12" s="27" t="n">
         <f aca="false">ROUND(G12,-2)</f>
-        <v>12800</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="17" t="s">
+        <v>10200</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B13" s="18" t="s">
         <v>47</v>
       </c>
-      <c r="C13" s="26" t="n">
+      <c r="C13" s="27" t="n">
         <f aca="false">H7</f>
         <v>7100</v>
       </c>
-      <c r="D13" s="27" t="n">
+      <c r="D13" s="28" t="n">
         <f aca="false">(H7/C7)^(1/10)-1</f>
         <v>-0.0118637399993557</v>
       </c>
-      <c r="E13" s="27" t="n">
+      <c r="E13" s="28" t="n">
         <f aca="false">(H7/E7)^(1/6)-1</f>
         <v>0.0072213107942356</v>
       </c>
-      <c r="F13" s="28" t="n">
+      <c r="F13" s="29" t="n">
         <v>0.03</v>
       </c>
-      <c r="G13" s="26" t="n">
+      <c r="G13" s="27" t="n">
         <f aca="false">C13*(1+F13)^($D$16-2023)</f>
         <v>8230.84592753</v>
       </c>
-      <c r="H13" s="26" t="n">
+      <c r="H13" s="27" t="n">
         <f aca="false">ROUND(G13,-2)</f>
         <v>8200</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="17" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B15" s="18" t="s">
         <v>48</v>
       </c>
-      <c r="C15" s="22"/>
-      <c r="D15" s="29" t="n">
+      <c r="C15" s="23"/>
+      <c r="D15" s="30" t="n">
         <v>2027</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="17" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B16" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="C16" s="22"/>
-      <c r="D16" s="30" t="n">
+      <c r="C16" s="23"/>
+      <c r="D16" s="31" t="n">
         <f aca="false">D15+1</f>
         <v>2028</v>
       </c>
-      <c r="E16" s="20" t="s">
+      <c r="E16" s="21" t="s">
         <v>50</v>
       </c>
-      <c r="F16" s="20"/>
-      <c r="G16" s="20"/>
-      <c r="H16" s="20"/>
-      <c r="I16" s="20"/>
-      <c r="J16" s="20"/>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="24" t="s">
+      <c r="F16" s="21"/>
+      <c r="G16" s="21"/>
+      <c r="H16" s="21"/>
+      <c r="I16" s="21"/>
+      <c r="J16" s="21"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B19" s="25" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="17" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B20" s="18" t="s">
         <v>52</v>
       </c>
-      <c r="C20" s="22"/>
-      <c r="D20" s="31" t="n">
+      <c r="C20" s="23"/>
+      <c r="D20" s="32" t="n">
         <f aca="false">C12-C13</f>
-        <v>3900</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="17" t="s">
+        <v>1700</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B21" s="18" t="s">
         <v>53</v>
       </c>
-      <c r="C21" s="22"/>
-      <c r="D21" s="32" t="n">
+      <c r="C21" s="23"/>
+      <c r="D21" s="33" t="n">
         <f aca="false">ROUND(D20*(1+F12)^($D$16-2023),-2)</f>
-        <v>4500</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B24" s="33" t="s">
+      <c r="B24" s="34" t="s">
         <v>12</v>
       </c>
-      <c r="C24" s="33"/>
-      <c r="D24" s="33"/>
-      <c r="E24" s="33"/>
-      <c r="F24" s="33"/>
-      <c r="G24" s="33"/>
-      <c r="H24" s="33"/>
-      <c r="I24" s="33"/>
-      <c r="J24" s="33"/>
+      <c r="C24" s="34"/>
+      <c r="D24" s="34"/>
+      <c r="E24" s="34"/>
+      <c r="F24" s="34"/>
+      <c r="G24" s="34"/>
+      <c r="H24" s="34"/>
+      <c r="I24" s="34"/>
+      <c r="J24" s="34"/>
     </row>
     <row r="25" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B25" s="33" t="s">
+      <c r="B25" s="34" t="s">
         <v>54</v>
       </c>
-      <c r="C25" s="33"/>
-      <c r="D25" s="33"/>
-      <c r="E25" s="33"/>
-      <c r="F25" s="33"/>
-      <c r="G25" s="33"/>
-      <c r="H25" s="33"/>
-      <c r="I25" s="33"/>
-      <c r="J25" s="33"/>
+      <c r="C25" s="34"/>
+      <c r="D25" s="34"/>
+      <c r="E25" s="34"/>
+      <c r="F25" s="34"/>
+      <c r="G25" s="34"/>
+      <c r="H25" s="34"/>
+      <c r="I25" s="34"/>
+      <c r="J25" s="34"/>
     </row>
     <row r="26" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B26" s="33" t="s">
+      <c r="B26" s="34" t="s">
         <v>55</v>
       </c>
-      <c r="C26" s="33"/>
-      <c r="D26" s="33"/>
-      <c r="E26" s="33"/>
-      <c r="F26" s="33"/>
-      <c r="G26" s="33"/>
-      <c r="H26" s="33"/>
-      <c r="I26" s="33"/>
-      <c r="J26" s="33"/>
+      <c r="C26" s="34"/>
+      <c r="D26" s="34"/>
+      <c r="E26" s="34"/>
+      <c r="F26" s="34"/>
+      <c r="G26" s="34"/>
+      <c r="H26" s="34"/>
+      <c r="I26" s="34"/>
+      <c r="J26" s="34"/>
     </row>
     <row r="27" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B27" s="33" t="s">
+      <c r="B27" s="34" t="s">
         <v>56</v>
       </c>
-      <c r="C27" s="33"/>
-      <c r="D27" s="33"/>
-      <c r="E27" s="33"/>
-      <c r="F27" s="33"/>
-      <c r="G27" s="33"/>
-      <c r="H27" s="33"/>
-      <c r="I27" s="33"/>
-      <c r="J27" s="33"/>
+      <c r="C27" s="34"/>
+      <c r="D27" s="34"/>
+      <c r="E27" s="34"/>
+      <c r="F27" s="34"/>
+      <c r="G27" s="34"/>
+      <c r="H27" s="34"/>
+      <c r="I27" s="34"/>
+      <c r="J27" s="34"/>
     </row>
     <row r="28" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B28" s="33" t="s">
+      <c r="B28" s="34" t="s">
         <v>57</v>
       </c>
-      <c r="C28" s="33"/>
-      <c r="D28" s="33"/>
-      <c r="E28" s="33"/>
-      <c r="F28" s="33"/>
-      <c r="G28" s="33"/>
-      <c r="H28" s="33"/>
-      <c r="I28" s="33"/>
-      <c r="J28" s="33"/>
+      <c r="C28" s="34"/>
+      <c r="D28" s="34"/>
+      <c r="E28" s="34"/>
+      <c r="F28" s="34"/>
+      <c r="G28" s="34"/>
+      <c r="H28" s="34"/>
+      <c r="I28" s="34"/>
+      <c r="J28" s="34"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -1458,92 +1462,92 @@
   <dimension ref="B2:C13"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="75"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="75"/>
   </cols>
   <sheetData>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="34" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B2" s="35" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B4" s="24" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B4" s="25" t="s">
         <v>59</v>
       </c>
-      <c r="C4" s="14" t="s">
+      <c r="C4" s="15" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="24" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B5" s="25" t="s">
         <v>61</v>
       </c>
-      <c r="C5" s="14" t="s">
+      <c r="C5" s="15" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="24" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B6" s="25" t="s">
         <v>39</v>
       </c>
-      <c r="C6" s="14" t="s">
+      <c r="C6" s="15" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="24" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B7" s="25" t="s">
         <v>64</v>
       </c>
-      <c r="C7" s="14" t="s">
+      <c r="C7" s="15" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="24" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B8" s="25" t="s">
         <v>66</v>
       </c>
-      <c r="C8" s="14" t="s">
+      <c r="C8" s="15" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="24" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B9" s="25" t="s">
         <v>68</v>
       </c>
-      <c r="C9" s="14" t="s">
+      <c r="C9" s="15" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="24" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B10" s="25" t="s">
         <v>70</v>
       </c>
-      <c r="C10" s="14" t="s">
+      <c r="C10" s="15" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="24" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B11" s="25" t="s">
         <v>72</v>
       </c>
-      <c r="C11" s="14" t="s">
+      <c r="C11" s="15" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="24" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B12" s="25" t="s">
         <v>74</v>
       </c>
-      <c r="C12" s="14" t="s">
+      <c r="C12" s="15" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="24" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B13" s="25" t="s">
         <v>76</v>
       </c>
-      <c r="C13" s="14" t="s">
+      <c r="C13" s="15" t="s">
         <v>77</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Trim AADT sheet notes to essentials
Drop the 11,000 segment-layer reference and the long explanatory notes;
8,800 is simply the 2023 value. Notes reduced to source stations, input
marker, and the difference-method caveat.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017bgXFHUDEAABZN3aMvsVWj
</commit_message>
<xml_diff>
--- a/3905_Page_Rd_Trip_Generation/Trip_Generation_3905_Page_Rd_Durham_NC.xlsx
+++ b/3905_Page_Rd_Trip_Generation/Trip_Generation_3905_Page_Rd_Durham_NC.xlsx
@@ -14,7 +14,7 @@
     <sheet name="Dev" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm.Print_Area" vbProcedure="false">AADT!$B$2:$J$28</definedName>
+    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm.Print_Area" vbProcedure="false">AADT!$B$2:$J$27</definedName>
     <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">TripGen!$B$2:$K$11</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="77">
   <si>
     <t xml:space="preserve">Trip Generation Table - 12th Edition</t>
   </si>
@@ -131,7 +131,7 @@
     <t xml:space="preserve">2021</t>
   </si>
   <si>
-    <t xml:space="preserve">2023¹</t>
+    <t xml:space="preserve">2023</t>
   </si>
   <si>
     <t xml:space="preserve">Page Rd south of Airport Rd (0320000269)</t>
@@ -158,10 +158,10 @@
     <t xml:space="preserve">CAGR '17-'23</t>
   </si>
   <si>
-    <t xml:space="preserve">Selected Rate²</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Build AADT³</t>
+    <t xml:space="preserve">Selected Rate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Build AADT</t>
   </si>
   <si>
     <t xml:space="preserve">Build AADT (rounded)</t>
@@ -191,16 +191,13 @@
     <t xml:space="preserve">Projected to Build year at selected rate (south leg)</t>
   </si>
   <si>
-    <t xml:space="preserve">1. AADT history from the NCDOT AADT station layer (ncdot.maps.arcgis.com, retrieved August 2026): stations 0320000269 (Page Rd south of Airport Rd) and 0320000260 (Page Rd north of Airport Rd). Note: the NCDOT AADT traffic segment layer (Route 40001973032, MP 3.334-3.620, source "Maintenance") displays 11,000 vpd for the segment south of Airport Rd versus the 8,800 station history value; the published station count history is used here. The north segment (MP 2.728-3.334) matches its station history (7,100 vpd).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2. Selected growth rate is an engineering input (blue). Computed CAGRs bracket it: south leg 2.8% (2013-2023) / -1.9% (2017-2023); north leg -1.2% (2013-2023) / 0.7% (2017-2023). 3.0%/yr compounded is applied corridor-wide as a conservative planning rate above the observed long-term trend at both stations.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3. Build AADT = 2023 AADT x (1 + selected rate)^(Build year - 2023). Build year per City of Durham TIA Guidelines (durhamnc.gov, "Guidelines for Traffic Impact Analysis (TIA) Requirement"): the analysis must examine expected traffic conditions one year after the project is scheduled to be complete; with an assumed 2027 opening, Build year = 2028.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4. Difference method: the volume change between the two Page Rd legs equals the net traffic exchanged with Airport Rd at the intersection. It is a LOWER-BOUND estimate of Airport Rd AADT - actual Airport Rd AADT = (11,000 + 7,100) - 2 x (Page Rd through volume), which cannot be isolated from AADT data alone. Verify with the project turning movement count.</t>
+    <t xml:space="preserve">1. Source: NCDOT AADT stations 0320000269 (Page Rd south of Airport Rd) and 0320000260 (Page Rd north of Airport Rd), ncdot.maps.arcgis.com.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. Selected growth rate is an input (blue cells).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. Difference method is a minimum estimate of Airport Rd volume; verify with the project TMC.</t>
   </si>
   <si>
     <t xml:space="preserve">Development Summary</t>
@@ -466,7 +463,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="37">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -604,6 +601,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1382,7 +1383,7 @@
       <c r="I24" s="34"/>
       <c r="J24" s="34"/>
     </row>
-    <row r="25" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B25" s="34" t="s">
         <v>54</v>
       </c>
@@ -1395,7 +1396,7 @@
       <c r="I25" s="34"/>
       <c r="J25" s="34"/>
     </row>
-    <row r="26" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B26" s="34" t="s">
         <v>55</v>
       </c>
@@ -1408,7 +1409,7 @@
       <c r="I26" s="34"/>
       <c r="J26" s="34"/>
     </row>
-    <row r="27" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B27" s="34" t="s">
         <v>56</v>
       </c>
@@ -1422,27 +1423,16 @@
       <c r="J27" s="34"/>
     </row>
     <row r="28" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B28" s="34" t="s">
-        <v>57</v>
-      </c>
-      <c r="C28" s="34"/>
-      <c r="D28" s="34"/>
-      <c r="E28" s="34"/>
-      <c r="F28" s="34"/>
-      <c r="G28" s="34"/>
-      <c r="H28" s="34"/>
-      <c r="I28" s="34"/>
-      <c r="J28" s="34"/>
+      <c r="B28" s="35"/>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="6">
     <mergeCell ref="B2:J2"/>
     <mergeCell ref="E16:J16"/>
     <mergeCell ref="B24:J24"/>
     <mergeCell ref="B25:J25"/>
     <mergeCell ref="B26:J26"/>
     <mergeCell ref="B27:J27"/>
-    <mergeCell ref="B28:J28"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1467,24 +1457,24 @@
   </cols>
   <sheetData>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B2" s="35" t="s">
-        <v>58</v>
+      <c r="B2" s="36" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="25" t="s">
+        <v>58</v>
+      </c>
+      <c r="C4" s="15" t="s">
         <v>59</v>
-      </c>
-      <c r="C4" s="15" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="25" t="s">
+        <v>60</v>
+      </c>
+      <c r="C5" s="15" t="s">
         <v>61</v>
-      </c>
-      <c r="C5" s="15" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1492,63 +1482,63 @@
         <v>39</v>
       </c>
       <c r="C6" s="15" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="25" t="s">
+        <v>63</v>
+      </c>
+      <c r="C7" s="15" t="s">
         <v>64</v>
-      </c>
-      <c r="C7" s="15" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B8" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="C8" s="15" t="s">
         <v>66</v>
-      </c>
-      <c r="C8" s="15" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B9" s="25" t="s">
+        <v>67</v>
+      </c>
+      <c r="C9" s="15" t="s">
         <v>68</v>
-      </c>
-      <c r="C9" s="15" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="25" t="s">
+        <v>69</v>
+      </c>
+      <c r="C10" s="15" t="s">
         <v>70</v>
-      </c>
-      <c r="C10" s="15" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B11" s="25" t="s">
+        <v>71</v>
+      </c>
+      <c r="C11" s="15" t="s">
         <v>72</v>
-      </c>
-      <c r="C11" s="15" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="25" t="s">
+        <v>73</v>
+      </c>
+      <c r="C12" s="15" t="s">
         <v>74</v>
-      </c>
-      <c r="C12" s="15" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B13" s="25" t="s">
+        <v>75</v>
+      </c>
+      <c r="C13" s="15" t="s">
         <v>76</v>
-      </c>
-      <c r="C13" s="15" t="s">
-        <v>77</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add draft turn lane evaluation figures and site trip assignment
Three pre-count figures (access/lane configuration, draft directional
distribution, AM/PM site trip assignment) reflecting: RIRO at both Page
Road driveways, auto driveways (upper Page, west Airport) carrying peak
hour trips, truck driveways (lower Page, east Airport) negligible in
peaks. New Assign sheet computes movement-level volumes from a blue
35/25/40 distribution input, balancing exactly to the 62/10 AM and
18/56 PM control totals. Airport Rd corridor AADT treated as
unpublished pending the TMC; NC-540 ramp volumes (7,600 / 3,500 at
Pleasant Grove Church Rd) retained as reference inputs only.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017bgXFHUDEAABZN3aMvsVWj
</commit_message>
<xml_diff>
--- a/3905_Page_Rd_Trip_Generation/Trip_Generation_3905_Page_Rd_Durham_NC.xlsx
+++ b/3905_Page_Rd_Trip_Generation/Trip_Generation_3905_Page_Rd_Durham_NC.xlsx
@@ -10,11 +10,13 @@
   <sheets>
     <sheet name="TripGen" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Rates" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="AADT" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="Dev" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Assign" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="AADT" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Dev" sheetId="5" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm.Print_Area" vbProcedure="false">AADT!$B$2:$J$27</definedName>
+    <definedName function="false" hidden="false" localSheetId="3" name="_xlnm.Print_Area" vbProcedure="false">AADT!$B$2:$J$27</definedName>
+    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm.Print_Area" vbProcedure="false">Assign!$B$2:$H$29</definedName>
     <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">TripGen!$B$2:$K$11</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
@@ -27,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="112">
   <si>
     <t xml:space="preserve">Trip Generation Table - 12th Edition</t>
   </si>
@@ -107,6 +109,108 @@
     <t xml:space="preserve">Result</t>
   </si>
   <si>
+    <t xml:space="preserve">Draft Site Trip Assignment - Turn Lane Evaluation (pre-count)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Directional Distribution (blue inputs; draft, AADT-weighted)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">To/from south via Page Rd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">To/from north via Page Rd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">To/from southeast via Airport Rd / Pleasant Grove Church Rd (NC-540)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Peak Hour Site Trips (from TripGen)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AM In</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AM Out</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PM In</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PM Out</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Control totals</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Driveway Movement Assignment</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Access / Movement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Serves</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Share</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Page Rd Dwy (auto, RIRO): NB right-in</t>
+  </si>
+  <si>
+    <t xml:space="preserve">From south</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Page Rd Dwy (auto, RIRO): right-out to north</t>
+  </si>
+  <si>
+    <t xml:space="preserve">To north</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Airport Rd Dwy (auto): EB right-in</t>
+  </si>
+  <si>
+    <t xml:space="preserve">From north (via int.)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Airport Rd Dwy (auto): WB left-in</t>
+  </si>
+  <si>
+    <t xml:space="preserve">From SE (NC-540)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Airport Rd Dwy (auto): WB left-out (to south via int.)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">To south</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Airport Rd Dwy (auto): EB right-out</t>
+  </si>
+  <si>
+    <t xml:space="preserve">To SE (NC-540)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Truck driveways (Page Rd S dwy / Airport Rd E dwy)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trucks, off-peak</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Distribution is a draft engineering input pending the TMC; based on relative background volumes on Page Rd (8,800 S / 7,100 N, 2023) and regional access (I-40 via Page Rd south; NC-540 via Pleasant Grove Church Rd southeast).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. Peak hour trips assigned to the two auto driveways; truck driveways assumed negligible during peak hours.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. Page Rd driveways assumed right-in/right-out only; Airport Rd driveways assumed full movement. Arrivals from the north and departures to the south route through the Page Rd / Airport Rd intersection.</t>
+  </si>
+  <si>
     <t xml:space="preserve">NCDOT AADT Data &amp; Growth Projections - Page Road (SR 1973)</t>
   </si>
   <si>
@@ -137,9 +241,6 @@
     <t xml:space="preserve">Page Rd south of Airport Rd (0320000269)</t>
   </si>
   <si>
-    <t xml:space="preserve">-</t>
-  </si>
-  <si>
     <t xml:space="preserve">Page Rd north of Airport Rd (0320000260)</t>
   </si>
   <si>
@@ -182,13 +283,19 @@
     <t xml:space="preserve">Per City of Durham TIA Guidelines: analysis examines conditions one year after project completion</t>
   </si>
   <si>
-    <t xml:space="preserve">Airport Road (SR 1971) AADT Estimate - Difference Method</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Page Rd S of Airport Rd minus N of Airport Rd (2023)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Projected to Build year at selected rate (south leg)</t>
+    <t xml:space="preserve">Airport Rd / Pleasant Grove Church Rd Corridor (no published AADT)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Difference method at Page Rd intersection (minimum)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NC-540 ramps at Pleasant Grove Church Rd (reference, blue inputs)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Corridor AADT at site frontage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pending TMC</t>
   </si>
   <si>
     <t xml:space="preserve">1. Source: NCDOT AADT stations 0320000269 (Page Rd south of Airport Rd) and 0320000260 (Page Rd north of Airport Rd), ncdot.maps.arcgis.com.</t>
@@ -197,7 +304,7 @@
     <t xml:space="preserve">2. Selected growth rate is an input (blue cells).</t>
   </si>
   <si>
-    <t xml:space="preserve">3. Difference method is a minimum estimate of Airport Rd volume; verify with the project TMC.</t>
+    <t xml:space="preserve">3. Corridor AADT is not published. Difference method is a minimum at the Page Rd leg; the NC-540 ramp total (no ramp-to-ramp assumed) exchanges with the corridor but its split toward the site vs. southeast is unknown. Confirm with the project TMC.</t>
   </si>
   <si>
     <t xml:space="preserve">Development Summary</t>
@@ -463,7 +570,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="41">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -568,6 +675,30 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="168" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="166" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -589,14 +720,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="171" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1138,6 +1261,411 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
+  <dimension ref="B2:H29"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="2.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="5" style="1" width="9"/>
+  </cols>
+  <sheetData>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B2" s="16" t="s">
+        <v>26</v>
+      </c>
+      <c r="C2" s="16"/>
+      <c r="D2" s="16"/>
+      <c r="E2" s="16"/>
+      <c r="F2" s="16"/>
+      <c r="G2" s="16"/>
+      <c r="H2" s="16"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B4" s="25" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B5" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" s="23"/>
+      <c r="D5" s="20" t="n">
+        <v>0.35</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B6" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="C6" s="23"/>
+      <c r="D6" s="20" t="n">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B7" s="18" t="s">
+        <v>30</v>
+      </c>
+      <c r="C7" s="23"/>
+      <c r="D7" s="20" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B8" s="18" t="s">
+        <v>31</v>
+      </c>
+      <c r="C8" s="23"/>
+      <c r="D8" s="26" t="n">
+        <f aca="false">SUM(D5:D7)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B10" s="25" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B11" s="23"/>
+      <c r="C11" s="23"/>
+      <c r="D11" s="23"/>
+      <c r="E11" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="F11" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="G11" s="17" t="s">
+        <v>35</v>
+      </c>
+      <c r="H11" s="17" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B12" s="18" t="s">
+        <v>37</v>
+      </c>
+      <c r="C12" s="23"/>
+      <c r="D12" s="23"/>
+      <c r="E12" s="27" t="n">
+        <f aca="false">TripGen!F7</f>
+        <v>62</v>
+      </c>
+      <c r="F12" s="27" t="n">
+        <f aca="false">TripGen!G7</f>
+        <v>10</v>
+      </c>
+      <c r="G12" s="27" t="n">
+        <f aca="false">TripGen!I7</f>
+        <v>18</v>
+      </c>
+      <c r="H12" s="27" t="n">
+        <f aca="false">TripGen!J7</f>
+        <v>56</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B15" s="25" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B16" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="C16" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="D16" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="E16" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="F16" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="G16" s="17" t="s">
+        <v>35</v>
+      </c>
+      <c r="H16" s="17" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B17" s="18" t="s">
+        <v>42</v>
+      </c>
+      <c r="C17" s="24" t="s">
+        <v>43</v>
+      </c>
+      <c r="D17" s="28" t="n">
+        <f aca="false">D5</f>
+        <v>0.35</v>
+      </c>
+      <c r="E17" s="27" t="n">
+        <f aca="false">ROUND(D17*$E$12,0)</f>
+        <v>22</v>
+      </c>
+      <c r="F17" s="27" t="s">
+        <v>44</v>
+      </c>
+      <c r="G17" s="27" t="n">
+        <f aca="false">ROUND(D17*$G$12,0)</f>
+        <v>6</v>
+      </c>
+      <c r="H17" s="27" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B18" s="18" t="s">
+        <v>45</v>
+      </c>
+      <c r="C18" s="24" t="s">
+        <v>46</v>
+      </c>
+      <c r="D18" s="28" t="n">
+        <f aca="false">D6</f>
+        <v>0.25</v>
+      </c>
+      <c r="E18" s="27" t="s">
+        <v>44</v>
+      </c>
+      <c r="F18" s="27" t="n">
+        <f aca="false">ROUND(D18*$F$12,0)</f>
+        <v>3</v>
+      </c>
+      <c r="G18" s="27" t="s">
+        <v>44</v>
+      </c>
+      <c r="H18" s="27" t="n">
+        <f aca="false">ROUND(D18*$H$12,0)</f>
+        <v>14</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B19" s="18" t="s">
+        <v>47</v>
+      </c>
+      <c r="C19" s="24" t="s">
+        <v>48</v>
+      </c>
+      <c r="D19" s="28" t="n">
+        <f aca="false">D6</f>
+        <v>0.25</v>
+      </c>
+      <c r="E19" s="27" t="n">
+        <f aca="false">ROUND(D19*$E$12,0)</f>
+        <v>16</v>
+      </c>
+      <c r="F19" s="27" t="s">
+        <v>44</v>
+      </c>
+      <c r="G19" s="27" t="n">
+        <f aca="false">ROUND(D19*$G$12,0)</f>
+        <v>5</v>
+      </c>
+      <c r="H19" s="27" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B20" s="18" t="s">
+        <v>49</v>
+      </c>
+      <c r="C20" s="24" t="s">
+        <v>50</v>
+      </c>
+      <c r="D20" s="28" t="n">
+        <f aca="false">D7</f>
+        <v>0.4</v>
+      </c>
+      <c r="E20" s="27" t="n">
+        <f aca="false">$E$12-E17-E19</f>
+        <v>24</v>
+      </c>
+      <c r="F20" s="27" t="s">
+        <v>44</v>
+      </c>
+      <c r="G20" s="27" t="n">
+        <f aca="false">$G$12-G17-G19</f>
+        <v>7</v>
+      </c>
+      <c r="H20" s="27" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B21" s="18" t="s">
+        <v>51</v>
+      </c>
+      <c r="C21" s="24" t="s">
+        <v>52</v>
+      </c>
+      <c r="D21" s="28" t="n">
+        <f aca="false">D5</f>
+        <v>0.35</v>
+      </c>
+      <c r="E21" s="27" t="s">
+        <v>44</v>
+      </c>
+      <c r="F21" s="27" t="n">
+        <f aca="false">ROUND(D21*$F$12,0)</f>
+        <v>4</v>
+      </c>
+      <c r="G21" s="27" t="s">
+        <v>44</v>
+      </c>
+      <c r="H21" s="27" t="n">
+        <f aca="false">ROUND(D21*$H$12,0)</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B22" s="18" t="s">
+        <v>53</v>
+      </c>
+      <c r="C22" s="24" t="s">
+        <v>54</v>
+      </c>
+      <c r="D22" s="28" t="n">
+        <f aca="false">D7</f>
+        <v>0.4</v>
+      </c>
+      <c r="E22" s="27" t="s">
+        <v>44</v>
+      </c>
+      <c r="F22" s="27" t="n">
+        <f aca="false">$F$12-F18-F21</f>
+        <v>3</v>
+      </c>
+      <c r="G22" s="27" t="s">
+        <v>44</v>
+      </c>
+      <c r="H22" s="27" t="n">
+        <f aca="false">$H$12-H18-H21</f>
+        <v>22</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B23" s="18" t="s">
+        <v>55</v>
+      </c>
+      <c r="C23" s="24" t="s">
+        <v>56</v>
+      </c>
+      <c r="D23" s="24" t="s">
+        <v>44</v>
+      </c>
+      <c r="E23" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" s="27" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B24" s="29" t="s">
+        <v>9</v>
+      </c>
+      <c r="C24" s="23"/>
+      <c r="D24" s="23"/>
+      <c r="E24" s="30" t="n">
+        <f aca="false">SUM(E17:E23)</f>
+        <v>62</v>
+      </c>
+      <c r="F24" s="30" t="n">
+        <f aca="false">SUM(F17:F23)</f>
+        <v>10</v>
+      </c>
+      <c r="G24" s="30" t="n">
+        <f aca="false">SUM(G17:G23)</f>
+        <v>18</v>
+      </c>
+      <c r="H24" s="30" t="n">
+        <f aca="false">SUM(H17:H23)</f>
+        <v>56</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B26" s="31" t="s">
+        <v>12</v>
+      </c>
+      <c r="C26" s="31"/>
+      <c r="D26" s="31"/>
+      <c r="E26" s="31"/>
+      <c r="F26" s="31"/>
+      <c r="G26" s="31"/>
+      <c r="H26" s="31"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B27" s="31" t="s">
+        <v>57</v>
+      </c>
+      <c r="C27" s="31"/>
+      <c r="D27" s="31"/>
+      <c r="E27" s="31"/>
+      <c r="F27" s="31"/>
+      <c r="G27" s="31"/>
+      <c r="H27" s="31"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B28" s="31" t="s">
+        <v>58</v>
+      </c>
+      <c r="C28" s="31"/>
+      <c r="D28" s="31"/>
+      <c r="E28" s="31"/>
+      <c r="F28" s="31"/>
+      <c r="G28" s="31"/>
+      <c r="H28" s="31"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B29" s="31" t="s">
+        <v>59</v>
+      </c>
+      <c r="C29" s="31"/>
+      <c r="D29" s="31"/>
+      <c r="E29" s="31"/>
+      <c r="F29" s="31"/>
+      <c r="G29" s="31"/>
+      <c r="H29" s="31"/>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="B2:H2"/>
+    <mergeCell ref="B26:H26"/>
+    <mergeCell ref="B27:H27"/>
+    <mergeCell ref="B28:H28"/>
+    <mergeCell ref="B29:H29"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="true"/>
+  </sheetPr>
   <dimension ref="B2:J28"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -1149,7 +1677,7 @@
   <sheetData>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="16" t="s">
-        <v>26</v>
+        <v>60</v>
       </c>
       <c r="C2" s="16"/>
       <c r="D2" s="16"/>
@@ -1162,182 +1690,182 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="25" t="s">
-        <v>27</v>
+        <v>61</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="17" t="s">
-        <v>28</v>
+        <v>62</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>29</v>
+        <v>63</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>30</v>
+        <v>64</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>31</v>
+        <v>65</v>
       </c>
       <c r="F5" s="17" t="s">
-        <v>32</v>
+        <v>66</v>
       </c>
       <c r="G5" s="17" t="s">
-        <v>33</v>
+        <v>67</v>
       </c>
       <c r="H5" s="17" t="s">
-        <v>34</v>
+        <v>68</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="18" t="s">
-        <v>35</v>
-      </c>
-      <c r="C6" s="26" t="n">
+        <v>69</v>
+      </c>
+      <c r="C6" s="32" t="n">
         <v>6700</v>
       </c>
-      <c r="D6" s="26" t="n">
+      <c r="D6" s="32" t="n">
         <v>7700</v>
       </c>
-      <c r="E6" s="26" t="n">
+      <c r="E6" s="32" t="n">
         <v>9900</v>
       </c>
       <c r="F6" s="24" t="s">
-        <v>36</v>
-      </c>
-      <c r="G6" s="26" t="n">
+        <v>44</v>
+      </c>
+      <c r="G6" s="32" t="n">
         <v>10000</v>
       </c>
-      <c r="H6" s="26" t="n">
+      <c r="H6" s="32" t="n">
         <v>8800</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="18" t="s">
-        <v>37</v>
-      </c>
-      <c r="C7" s="26" t="n">
+        <v>70</v>
+      </c>
+      <c r="C7" s="32" t="n">
         <v>8000</v>
       </c>
-      <c r="D7" s="26" t="n">
+      <c r="D7" s="32" t="n">
         <v>5500</v>
       </c>
-      <c r="E7" s="26" t="n">
+      <c r="E7" s="32" t="n">
         <v>6800</v>
       </c>
-      <c r="F7" s="26" t="n">
+      <c r="F7" s="32" t="n">
         <v>8200</v>
       </c>
-      <c r="G7" s="26" t="n">
+      <c r="G7" s="32" t="n">
         <v>6600</v>
       </c>
-      <c r="H7" s="26" t="n">
+      <c r="H7" s="32" t="n">
         <v>7100</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="25" t="s">
-        <v>38</v>
+        <v>71</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B11" s="17" t="s">
-        <v>39</v>
+        <v>72</v>
       </c>
       <c r="C11" s="17" t="s">
-        <v>40</v>
+        <v>73</v>
       </c>
       <c r="D11" s="17" t="s">
-        <v>41</v>
+        <v>74</v>
       </c>
       <c r="E11" s="17" t="s">
-        <v>42</v>
+        <v>75</v>
       </c>
       <c r="F11" s="17" t="s">
-        <v>43</v>
+        <v>76</v>
       </c>
       <c r="G11" s="17" t="s">
-        <v>44</v>
+        <v>77</v>
       </c>
       <c r="H11" s="17" t="s">
-        <v>45</v>
+        <v>78</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="18" t="s">
-        <v>46</v>
-      </c>
-      <c r="C12" s="27" t="n">
+        <v>79</v>
+      </c>
+      <c r="C12" s="33" t="n">
         <f aca="false">H6</f>
         <v>8800</v>
       </c>
-      <c r="D12" s="28" t="n">
+      <c r="D12" s="34" t="n">
         <f aca="false">(H6/C6)^(1/10)-1</f>
         <v>0.0276394947719256</v>
       </c>
-      <c r="E12" s="28" t="n">
+      <c r="E12" s="34" t="n">
         <f aca="false">(H6/E6)^(1/6)-1</f>
         <v>-0.01943908218904</v>
       </c>
-      <c r="F12" s="29" t="n">
+      <c r="F12" s="35" t="n">
         <v>0.03</v>
       </c>
-      <c r="G12" s="27" t="n">
+      <c r="G12" s="33" t="n">
         <f aca="false">C12*(1+F12)^($D$16-2023)</f>
         <v>10201.61185384</v>
       </c>
-      <c r="H12" s="27" t="n">
+      <c r="H12" s="33" t="n">
         <f aca="false">ROUND(G12,-2)</f>
         <v>10200</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B13" s="18" t="s">
-        <v>47</v>
-      </c>
-      <c r="C13" s="27" t="n">
+        <v>80</v>
+      </c>
+      <c r="C13" s="33" t="n">
         <f aca="false">H7</f>
         <v>7100</v>
       </c>
-      <c r="D13" s="28" t="n">
+      <c r="D13" s="34" t="n">
         <f aca="false">(H7/C7)^(1/10)-1</f>
         <v>-0.0118637399993557</v>
       </c>
-      <c r="E13" s="28" t="n">
+      <c r="E13" s="34" t="n">
         <f aca="false">(H7/E7)^(1/6)-1</f>
         <v>0.0072213107942356</v>
       </c>
-      <c r="F13" s="29" t="n">
+      <c r="F13" s="35" t="n">
         <v>0.03</v>
       </c>
-      <c r="G13" s="27" t="n">
+      <c r="G13" s="33" t="n">
         <f aca="false">C13*(1+F13)^($D$16-2023)</f>
         <v>8230.84592753</v>
       </c>
-      <c r="H13" s="27" t="n">
+      <c r="H13" s="33" t="n">
         <f aca="false">ROUND(G13,-2)</f>
         <v>8200</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B15" s="18" t="s">
-        <v>48</v>
+        <v>81</v>
       </c>
       <c r="C15" s="23"/>
-      <c r="D15" s="30" t="n">
+      <c r="D15" s="36" t="n">
         <v>2027</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B16" s="18" t="s">
-        <v>49</v>
+        <v>82</v>
       </c>
       <c r="C16" s="23"/>
-      <c r="D16" s="31" t="n">
+      <c r="D16" s="37" t="n">
         <f aca="false">D15+1</f>
         <v>2028</v>
       </c>
       <c r="E16" s="21" t="s">
-        <v>50</v>
+        <v>83</v>
       </c>
       <c r="F16" s="21"/>
       <c r="G16" s="21"/>
@@ -1347,83 +1875,98 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B19" s="25" t="s">
-        <v>51</v>
+        <v>84</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B20" s="18" t="s">
-        <v>52</v>
+        <v>85</v>
       </c>
       <c r="C20" s="23"/>
-      <c r="D20" s="32" t="n">
+      <c r="D20" s="27" t="n">
         <f aca="false">C12-C13</f>
         <v>1700</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B21" s="18" t="s">
-        <v>53</v>
+        <v>86</v>
       </c>
       <c r="C21" s="23"/>
-      <c r="D21" s="33" t="n">
-        <f aca="false">ROUND(D20*(1+F12)^($D$16-2023),-2)</f>
-        <v>2000</v>
+      <c r="D21" s="30" t="n">
+        <f aca="false">F21+G21</f>
+        <v>11100</v>
+      </c>
+      <c r="F21" s="32" t="n">
+        <v>7600</v>
+      </c>
+      <c r="G21" s="32" t="n">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B22" s="18" t="s">
+        <v>87</v>
+      </c>
+      <c r="C22" s="23"/>
+      <c r="D22" s="30" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B24" s="34" t="s">
+      <c r="B24" s="38" t="s">
         <v>12</v>
       </c>
-      <c r="C24" s="34"/>
-      <c r="D24" s="34"/>
-      <c r="E24" s="34"/>
-      <c r="F24" s="34"/>
-      <c r="G24" s="34"/>
-      <c r="H24" s="34"/>
-      <c r="I24" s="34"/>
-      <c r="J24" s="34"/>
+      <c r="C24" s="38"/>
+      <c r="D24" s="38"/>
+      <c r="E24" s="38"/>
+      <c r="F24" s="38"/>
+      <c r="G24" s="38"/>
+      <c r="H24" s="38"/>
+      <c r="I24" s="38"/>
+      <c r="J24" s="38"/>
     </row>
     <row r="25" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B25" s="34" t="s">
-        <v>54</v>
-      </c>
-      <c r="C25" s="34"/>
-      <c r="D25" s="34"/>
-      <c r="E25" s="34"/>
-      <c r="F25" s="34"/>
-      <c r="G25" s="34"/>
-      <c r="H25" s="34"/>
-      <c r="I25" s="34"/>
-      <c r="J25" s="34"/>
+      <c r="B25" s="38" t="s">
+        <v>89</v>
+      </c>
+      <c r="C25" s="38"/>
+      <c r="D25" s="38"/>
+      <c r="E25" s="38"/>
+      <c r="F25" s="38"/>
+      <c r="G25" s="38"/>
+      <c r="H25" s="38"/>
+      <c r="I25" s="38"/>
+      <c r="J25" s="38"/>
     </row>
     <row r="26" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B26" s="34" t="s">
-        <v>55</v>
-      </c>
-      <c r="C26" s="34"/>
-      <c r="D26" s="34"/>
-      <c r="E26" s="34"/>
-      <c r="F26" s="34"/>
-      <c r="G26" s="34"/>
-      <c r="H26" s="34"/>
-      <c r="I26" s="34"/>
-      <c r="J26" s="34"/>
+      <c r="B26" s="38" t="s">
+        <v>90</v>
+      </c>
+      <c r="C26" s="38"/>
+      <c r="D26" s="38"/>
+      <c r="E26" s="38"/>
+      <c r="F26" s="38"/>
+      <c r="G26" s="38"/>
+      <c r="H26" s="38"/>
+      <c r="I26" s="38"/>
+      <c r="J26" s="38"/>
     </row>
     <row r="27" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B27" s="34" t="s">
-        <v>56</v>
-      </c>
-      <c r="C27" s="34"/>
-      <c r="D27" s="34"/>
-      <c r="E27" s="34"/>
-      <c r="F27" s="34"/>
-      <c r="G27" s="34"/>
-      <c r="H27" s="34"/>
-      <c r="I27" s="34"/>
-      <c r="J27" s="34"/>
+      <c r="B27" s="38" t="s">
+        <v>91</v>
+      </c>
+      <c r="C27" s="38"/>
+      <c r="D27" s="38"/>
+      <c r="E27" s="38"/>
+      <c r="F27" s="38"/>
+      <c r="G27" s="38"/>
+      <c r="H27" s="38"/>
+      <c r="I27" s="38"/>
+      <c r="J27" s="38"/>
     </row>
     <row r="28" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B28" s="35"/>
+      <c r="B28" s="39"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -1444,7 +1987,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -1457,88 +2000,88 @@
   </cols>
   <sheetData>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B2" s="36" t="s">
-        <v>57</v>
+      <c r="B2" s="40" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="25" t="s">
-        <v>58</v>
+        <v>93</v>
       </c>
       <c r="C4" s="15" t="s">
-        <v>59</v>
+        <v>94</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="25" t="s">
-        <v>60</v>
+        <v>95</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>61</v>
+        <v>96</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="25" t="s">
-        <v>39</v>
+        <v>72</v>
       </c>
       <c r="C6" s="15" t="s">
-        <v>62</v>
+        <v>97</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="25" t="s">
-        <v>63</v>
+        <v>98</v>
       </c>
       <c r="C7" s="15" t="s">
-        <v>64</v>
+        <v>99</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B8" s="25" t="s">
-        <v>65</v>
+        <v>100</v>
       </c>
       <c r="C8" s="15" t="s">
-        <v>66</v>
+        <v>101</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B9" s="25" t="s">
-        <v>67</v>
+        <v>102</v>
       </c>
       <c r="C9" s="15" t="s">
-        <v>68</v>
+        <v>103</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="25" t="s">
-        <v>69</v>
+        <v>104</v>
       </c>
       <c r="C10" s="15" t="s">
-        <v>70</v>
+        <v>105</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B11" s="25" t="s">
-        <v>71</v>
+        <v>106</v>
       </c>
       <c r="C11" s="15" t="s">
-        <v>72</v>
+        <v>107</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="25" t="s">
-        <v>73</v>
+        <v>108</v>
       </c>
       <c r="C12" s="15" t="s">
-        <v>74</v>
+        <v>109</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B13" s="25" t="s">
-        <v>75</v>
+        <v>110</v>
       </c>
       <c r="C13" s="15" t="s">
-        <v>76</v>
+        <v>111</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Use SR 1789 segment AADT for corridor; drop NC-540 ramp data
The NC-540 ramps pass under the Airport Rd / Pleasant Grove Church Rd
corridor with no connection, so their volumes are removed everywhere.
Corridor AADT now estimated from the SR 1789 (Pleasant Grove Church Rd)
segment: 9,100 vpd (2023, station 0920000468 near the SE end), with
station history 7,300 (2013) / 7,800 (2015) added and a 2.2% CAGR
computed. Draft distribution re-weighted proportional to the three legs
(8,800 / 7,100 / 9,100) to 35/30/35, figures and Assign sheet updated;
SE regional access corrected to Aviation Pkwy / I-40.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017bgXFHUDEAABZN3aMvsVWj
</commit_message>
<xml_diff>
--- a/3905_Page_Rd_Trip_Generation/Trip_Generation_3905_Page_Rd_Durham_NC.xlsx
+++ b/3905_Page_Rd_Trip_Generation/Trip_Generation_3905_Page_Rd_Durham_NC.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="113">
   <si>
     <t xml:space="preserve">Trip Generation Table - 12th Edition</t>
   </si>
@@ -121,7 +121,7 @@
     <t xml:space="preserve">To/from north via Page Rd</t>
   </si>
   <si>
-    <t xml:space="preserve">To/from southeast via Airport Rd / Pleasant Grove Church Rd (NC-540)</t>
+    <t xml:space="preserve">To/from southeast via Airport Rd / Pleasant Grove Church Rd (Aviation Pkwy / I-40)</t>
   </si>
   <si>
     <t xml:space="preserve">Sum</t>
@@ -181,7 +181,7 @@
     <t xml:space="preserve">Airport Rd Dwy (auto): WB left-in</t>
   </si>
   <si>
-    <t xml:space="preserve">From SE (NC-540)</t>
+    <t xml:space="preserve">From SE (via PGC Rd)</t>
   </si>
   <si>
     <t xml:space="preserve">Airport Rd Dwy (auto): WB left-out (to south via int.)</t>
@@ -193,7 +193,7 @@
     <t xml:space="preserve">Airport Rd Dwy (auto): EB right-out</t>
   </si>
   <si>
-    <t xml:space="preserve">To SE (NC-540)</t>
+    <t xml:space="preserve">To SE (via PGC Rd)</t>
   </si>
   <si>
     <t xml:space="preserve">Truck driveways (Page Rd S dwy / Airport Rd E dwy)</t>
@@ -202,7 +202,7 @@
     <t xml:space="preserve">Trucks, off-peak</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Distribution is a draft engineering input pending the TMC; based on relative background volumes on Page Rd (8,800 S / 7,100 N, 2023) and regional access (I-40 via Page Rd south; NC-540 via Pleasant Grove Church Rd southeast).</t>
+    <t xml:space="preserve">1. Distribution is a draft engineering input pending the TMC; proportional to background volumes (Page Rd S 8,800 / Page Rd N 7,100 / Airport Rd-PGC Rd corridor 9,100 vpd).</t>
   </si>
   <si>
     <t xml:space="preserve">2. Peak hour trips assigned to the two auto driveways; truck driveways assumed negligible during peak hours.</t>
@@ -244,6 +244,9 @@
     <t xml:space="preserve">Page Rd north of Airport Rd (0320000260)</t>
   </si>
   <si>
+    <t xml:space="preserve">Airport Rd / Pleasant Grove Church Rd (0920000468)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Growth Rates &amp; Build Year Projection</t>
   </si>
   <si>
@@ -274,6 +277,9 @@
     <t xml:space="preserve">Page Rd north of Airport Rd</t>
   </si>
   <si>
+    <t xml:space="preserve">Airport Rd / PGC Rd corridor (SR 1789)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Assumed opening year</t>
   </si>
   <si>
@@ -283,28 +289,25 @@
     <t xml:space="preserve">Per City of Durham TIA Guidelines: analysis examines conditions one year after project completion</t>
   </si>
   <si>
-    <t xml:space="preserve">Airport Rd / Pleasant Grove Church Rd Corridor (no published AADT)</t>
+    <t xml:space="preserve">Airport Rd / Pleasant Grove Church Rd Corridor Estimate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SR 1789 segment AADT near SE end of corridor (2023)</t>
   </si>
   <si>
     <t xml:space="preserve">Difference method at Page Rd intersection (minimum)</t>
   </si>
   <si>
-    <t xml:space="preserve">NC-540 ramps at Pleasant Grove Church Rd (reference, blue inputs)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Corridor AADT at site frontage</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pending TMC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Source: NCDOT AADT stations 0320000269 (Page Rd south of Airport Rd) and 0320000260 (Page Rd north of Airport Rd), ncdot.maps.arcgis.com.</t>
+    <t xml:space="preserve">Projected to Build year at selected rate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Source: NCDOT AADT stations 0320000269 (Page Rd south of Airport Rd), 0320000260 (Page Rd north of Airport Rd), and 0920000468 (SR 1789 / Pleasant Grove Church Rd, Wake Co.), ncdot.maps.arcgis.com.</t>
   </si>
   <si>
     <t xml:space="preserve">2. Selected growth rate is an input (blue cells).</t>
   </si>
   <si>
-    <t xml:space="preserve">3. Corridor AADT is not published. Difference method is a minimum at the Page Rd leg; the NC-540 ramp total (no ramp-to-ramp assumed) exchanges with the corridor but its split toward the site vs. southeast is unknown. Confirm with the project TMC.</t>
+    <t xml:space="preserve">3. Corridor estimate uses the SR 1789 segment AADT (9,100, 2023, source "Supplemental") near the SE end of the corridor; limited development between the segment and the site. Difference method at the Page Rd intersection is a minimum. Confirm with the project TMC.</t>
   </si>
   <si>
     <t xml:space="preserve">Development Summary</t>
@@ -570,7 +573,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="43">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -715,11 +718,19 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="170" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="171" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="171" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1302,7 +1313,7 @@
       </c>
       <c r="C6" s="23"/>
       <c r="D6" s="20" t="n">
-        <v>0.25</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1311,7 +1322,7 @@
       </c>
       <c r="C7" s="23"/>
       <c r="D7" s="20" t="n">
-        <v>0.4</v>
+        <v>0.35</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1432,7 +1443,7 @@
       </c>
       <c r="D18" s="28" t="n">
         <f aca="false">D6</f>
-        <v>0.25</v>
+        <v>0.3</v>
       </c>
       <c r="E18" s="27" t="s">
         <v>44</v>
@@ -1446,7 +1457,7 @@
       </c>
       <c r="H18" s="27" t="n">
         <f aca="false">ROUND(D18*$H$12,0)</f>
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1458,11 +1469,11 @@
       </c>
       <c r="D19" s="28" t="n">
         <f aca="false">D6</f>
-        <v>0.25</v>
+        <v>0.3</v>
       </c>
       <c r="E19" s="27" t="n">
         <f aca="false">ROUND(D19*$E$12,0)</f>
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="F19" s="27" t="s">
         <v>44</v>
@@ -1484,11 +1495,11 @@
       </c>
       <c r="D20" s="28" t="n">
         <f aca="false">D7</f>
-        <v>0.4</v>
+        <v>0.35</v>
       </c>
       <c r="E20" s="27" t="n">
         <f aca="false">$E$12-E17-E19</f>
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="F20" s="27" t="s">
         <v>44</v>
@@ -1536,7 +1547,7 @@
       </c>
       <c r="D22" s="28" t="n">
         <f aca="false">D7</f>
-        <v>0.4</v>
+        <v>0.35</v>
       </c>
       <c r="E22" s="27" t="s">
         <v>44</v>
@@ -1550,7 +1561,7 @@
       </c>
       <c r="H22" s="27" t="n">
         <f aca="false">$H$12-H18-H21</f>
-        <v>22</v>
+        <v>19</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1762,37 +1773,60 @@
         <v>7100</v>
       </c>
     </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B8" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="C8" s="32" t="n">
+        <v>7300</v>
+      </c>
+      <c r="D8" s="32" t="n">
+        <v>7800</v>
+      </c>
+      <c r="E8" s="24" t="s">
+        <v>44</v>
+      </c>
+      <c r="F8" s="24" t="s">
+        <v>44</v>
+      </c>
+      <c r="G8" s="24" t="s">
+        <v>44</v>
+      </c>
+      <c r="H8" s="32" t="n">
+        <v>9100</v>
+      </c>
+    </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="25" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B11" s="17" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C11" s="17" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D11" s="17" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E11" s="17" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F11" s="17" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="G11" s="17" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="H11" s="17" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="18" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C12" s="33" t="n">
         <f aca="false">H6</f>
@@ -1820,7 +1854,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B13" s="18" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C13" s="33" t="n">
         <f aca="false">H7</f>
@@ -1846,26 +1880,53 @@
         <v>8200</v>
       </c>
     </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B14" s="18" t="s">
+        <v>82</v>
+      </c>
+      <c r="C14" s="27" t="n">
+        <f aca="false">H8</f>
+        <v>9100</v>
+      </c>
+      <c r="D14" s="36" t="n">
+        <f aca="false">(H8/C8)^(1/10)-1</f>
+        <v>0.0222846817221405</v>
+      </c>
+      <c r="E14" s="24" t="s">
+        <v>44</v>
+      </c>
+      <c r="F14" s="35" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="G14" s="27" t="n">
+        <f aca="false">C14*(1+F14)^($D$16-2023)</f>
+        <v>10549.39407613</v>
+      </c>
+      <c r="H14" s="27" t="n">
+        <f aca="false">ROUND(G14,-2)</f>
+        <v>10500</v>
+      </c>
+    </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B15" s="18" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C15" s="23"/>
-      <c r="D15" s="36" t="n">
+      <c r="D15" s="37" t="n">
         <v>2027</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B16" s="18" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C16" s="23"/>
-      <c r="D16" s="37" t="n">
+      <c r="D16" s="38" t="n">
         <f aca="false">D15+1</f>
         <v>2028</v>
       </c>
       <c r="E16" s="21" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F16" s="21"/>
       <c r="G16" s="21"/>
@@ -1875,98 +1936,95 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B19" s="25" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B20" s="18" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C20" s="23"/>
-      <c r="D20" s="27" t="n">
+      <c r="D20" s="30" t="n">
+        <f aca="false">H8</f>
+        <v>9100</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B21" s="18" t="s">
+        <v>88</v>
+      </c>
+      <c r="C21" s="23"/>
+      <c r="D21" s="27" t="n">
         <f aca="false">C12-C13</f>
         <v>1700</v>
       </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B21" s="18" t="s">
-        <v>86</v>
-      </c>
-      <c r="C21" s="23"/>
-      <c r="D21" s="30" t="n">
-        <f aca="false">F21+G21</f>
-        <v>11100</v>
-      </c>
-      <c r="F21" s="32" t="n">
-        <v>7600</v>
-      </c>
-      <c r="G21" s="32" t="n">
-        <v>3500</v>
-      </c>
+      <c r="F21" s="39"/>
+      <c r="G21" s="39"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B22" s="18" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C22" s="23"/>
-      <c r="D22" s="30" t="s">
-        <v>88</v>
+      <c r="D22" s="27" t="n">
+        <f aca="false">ROUND(C14*(1+F14)^($D$16-2023),-2)</f>
+        <v>10500</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B24" s="38" t="s">
+      <c r="B24" s="40" t="s">
         <v>12</v>
       </c>
-      <c r="C24" s="38"/>
-      <c r="D24" s="38"/>
-      <c r="E24" s="38"/>
-      <c r="F24" s="38"/>
-      <c r="G24" s="38"/>
-      <c r="H24" s="38"/>
-      <c r="I24" s="38"/>
-      <c r="J24" s="38"/>
+      <c r="C24" s="40"/>
+      <c r="D24" s="40"/>
+      <c r="E24" s="40"/>
+      <c r="F24" s="40"/>
+      <c r="G24" s="40"/>
+      <c r="H24" s="40"/>
+      <c r="I24" s="40"/>
+      <c r="J24" s="40"/>
     </row>
     <row r="25" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B25" s="38" t="s">
-        <v>89</v>
-      </c>
-      <c r="C25" s="38"/>
-      <c r="D25" s="38"/>
-      <c r="E25" s="38"/>
-      <c r="F25" s="38"/>
-      <c r="G25" s="38"/>
-      <c r="H25" s="38"/>
-      <c r="I25" s="38"/>
-      <c r="J25" s="38"/>
+      <c r="B25" s="40" t="s">
+        <v>90</v>
+      </c>
+      <c r="C25" s="40"/>
+      <c r="D25" s="40"/>
+      <c r="E25" s="40"/>
+      <c r="F25" s="40"/>
+      <c r="G25" s="40"/>
+      <c r="H25" s="40"/>
+      <c r="I25" s="40"/>
+      <c r="J25" s="40"/>
     </row>
     <row r="26" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B26" s="38" t="s">
-        <v>90</v>
-      </c>
-      <c r="C26" s="38"/>
-      <c r="D26" s="38"/>
-      <c r="E26" s="38"/>
-      <c r="F26" s="38"/>
-      <c r="G26" s="38"/>
-      <c r="H26" s="38"/>
-      <c r="I26" s="38"/>
-      <c r="J26" s="38"/>
+      <c r="B26" s="40" t="s">
+        <v>91</v>
+      </c>
+      <c r="C26" s="40"/>
+      <c r="D26" s="40"/>
+      <c r="E26" s="40"/>
+      <c r="F26" s="40"/>
+      <c r="G26" s="40"/>
+      <c r="H26" s="40"/>
+      <c r="I26" s="40"/>
+      <c r="J26" s="40"/>
     </row>
     <row r="27" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B27" s="38" t="s">
-        <v>91</v>
-      </c>
-      <c r="C27" s="38"/>
-      <c r="D27" s="38"/>
-      <c r="E27" s="38"/>
-      <c r="F27" s="38"/>
-      <c r="G27" s="38"/>
-      <c r="H27" s="38"/>
-      <c r="I27" s="38"/>
-      <c r="J27" s="38"/>
+      <c r="B27" s="40" t="s">
+        <v>92</v>
+      </c>
+      <c r="C27" s="40"/>
+      <c r="D27" s="40"/>
+      <c r="E27" s="40"/>
+      <c r="F27" s="40"/>
+      <c r="G27" s="40"/>
+      <c r="H27" s="40"/>
+      <c r="I27" s="40"/>
+      <c r="J27" s="40"/>
     </row>
     <row r="28" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B28" s="39"/>
+      <c r="B28" s="41"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -2000,88 +2058,88 @@
   </cols>
   <sheetData>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B2" s="40" t="s">
-        <v>92</v>
+      <c r="B2" s="42" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="25" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C4" s="15" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="25" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="25" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C6" s="15" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="25" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C7" s="15" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B8" s="25" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C8" s="15" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B9" s="25" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C9" s="15" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="25" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C10" s="15" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B11" s="25" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C11" s="15" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="25" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C12" s="15" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B13" s="25" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C13" s="15" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Remove average-rates note and its table superscript
Drop note 2 ("Total site trips are determined based on the ITE average
rates") and the superscript 2 on the Total Site Trips band from both
the memo Table 1 and the workbook TripGen sheet; note 1 and the LUC
superscript remain.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017bgXFHUDEAABZN3aMvsVWj
</commit_message>
<xml_diff>
--- a/3905_Page_Rd_Trip_Generation/Trip_Generation_3905_Page_Rd_Durham_NC.xlsx
+++ b/3905_Page_Rd_Trip_Generation/Trip_Generation_3905_Page_Rd_Durham_NC.xlsx
@@ -10636,7 +10636,7 @@
     <row r="6" ht="18" customHeight="1" s="48">
       <c r="B6" s="61" t="inlineStr">
         <is>
-          <t>Total Site Trips²</t>
+          <t>Total Site Trips</t>
         </is>
       </c>
       <c r="C6" s="62" t="n"/>
@@ -10706,11 +10706,7 @@
       </c>
     </row>
     <row r="11" ht="18" customHeight="1" s="48">
-      <c r="B11" s="69" t="inlineStr">
-        <is>
-          <t>2. Total site trips are determined based on the ITE average rates</t>
-        </is>
-      </c>
+      <c r="B11" s="69"/>
     </row>
   </sheetData>
   <mergeCells count="8">

</xml_diff>